<commit_message>
even better micro perturbation
10/20/2025
</commit_message>
<xml_diff>
--- a/Raw Data/two forces micro perturbed (15 tirals)(tapered and cylindrical)/Validation(2.00to1.25)(3tendon).xlsx
+++ b/Raw Data/two forces micro perturbed (15 tirals)(tapered and cylindrical)/Validation(2.00to1.25)(3tendon).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/Raw Data/two forces micro perturbed (15 tirals)(tapered and cylindrical)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3723" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3A95A45-45A6-4717-89D1-86B978217194}"/>
+  <xr:revisionPtr revIDLastSave="3842" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E546ED1A-0214-4ADF-B7C5-2C0BC78FF731}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Proximal Validation" sheetId="12" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="49">
   <si>
     <t>Fx (N)</t>
   </si>
@@ -232,19 +232,26 @@
     <t>}</t>
   </si>
   <si>
-    <t>2.0 weight</t>
+    <t>2.0, 1Tx weight</t>
+  </si>
+  <si>
+    <t>2.0, 10Tx weight</t>
+  </si>
+  <si>
+    <t>2.0, 100Tx weight</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -283,15 +290,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -349,11 +349,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF6D6D"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -520,10 +515,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -547,6 +541,7 @@
     <xf numFmtId="1" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -598,18 +593,18 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
-    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -967,7 +962,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B763EDC-8536-442D-A8D3-F37978D4DE80}">
-  <dimension ref="A1:AC18"/>
+  <dimension ref="A1:AC19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -982,7 +977,8 @@
     <col min="12" max="13" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="17" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="21" max="23" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="25" width="8.140625" bestFit="1" customWidth="1"/>
@@ -991,43 +987,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="23" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="25" t="s">
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="S1" s="26"/>
-      <c r="T1" s="26"/>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
-      <c r="X1" s="27" t="s">
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="Y1" s="28"/>
-      <c r="Z1" s="28"/>
-      <c r="AA1" s="28"/>
-      <c r="AB1" s="28"/>
-      <c r="AC1" s="29"/>
+      <c r="Y1" s="29"/>
+      <c r="Z1" s="29"/>
+      <c r="AA1" s="29"/>
+      <c r="AB1" s="29"/>
+      <c r="AC1" s="30"/>
     </row>
     <row r="2" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2580,6 +2576,16 @@
       <c r="AA18" s="17"/>
       <c r="AB18" s="17"/>
       <c r="AC18" s="17"/>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="L19" s="13">
+        <f>AVERAGE(L3:L17)</f>
+        <v>-1.7737582442350691E-3</v>
+      </c>
+      <c r="R19" s="41">
+        <f>AVERAGE(R3:R17)</f>
+        <v>1.1673939140572688E-4</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2634,61 +2640,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="23" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="33" t="s">
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="S1" s="34"/>
-      <c r="T1" s="34"/>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
-      <c r="W1" s="34"/>
-      <c r="X1" s="34"/>
-      <c r="Y1" s="34"/>
-      <c r="Z1" s="34"/>
-      <c r="AA1" s="31" t="s">
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="35"/>
+      <c r="Y1" s="35"/>
+      <c r="Z1" s="35"/>
+      <c r="AA1" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-      <c r="AF1" s="31"/>
-      <c r="AG1" s="31"/>
-      <c r="AH1" s="31"/>
-      <c r="AI1" s="32" t="s">
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="32"/>
+      <c r="AD1" s="32"/>
+      <c r="AE1" s="32"/>
+      <c r="AF1" s="32"/>
+      <c r="AG1" s="32"/>
+      <c r="AH1" s="32"/>
+      <c r="AI1" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="AJ1" s="32"/>
-      <c r="AK1" s="32"/>
-      <c r="AL1" s="32"/>
-      <c r="AM1" s="32"/>
-      <c r="AN1" s="32"/>
-      <c r="AO1" s="32"/>
-      <c r="AP1" s="32"/>
-      <c r="AQ1" s="32"/>
-      <c r="AR1" s="32"/>
-      <c r="AS1" s="32"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="33"/>
+      <c r="AR1" s="33"/>
+      <c r="AS1" s="33"/>
     </row>
     <row r="2" spans="1:45" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2802,16 +2808,16 @@
       <c r="AK2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="AL2" s="30" t="s">
+      <c r="AL2" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AM2" s="30"/>
-      <c r="AN2" s="30"/>
-      <c r="AO2" s="30"/>
-      <c r="AP2" s="30"/>
-      <c r="AQ2" s="30"/>
-      <c r="AR2" s="30"/>
-      <c r="AS2" s="30"/>
+      <c r="AM2" s="31"/>
+      <c r="AN2" s="31"/>
+      <c r="AO2" s="31"/>
+      <c r="AP2" s="31"/>
+      <c r="AQ2" s="31"/>
+      <c r="AR2" s="31"/>
+      <c r="AS2" s="31"/>
     </row>
     <row r="3" spans="1:45" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
@@ -2883,43 +2889,43 @@
         <v>0.41270199418067899</v>
       </c>
       <c r="R3" s="5">
-        <v>0.75348612182948604</v>
+        <v>0.76363365135228745</v>
       </c>
       <c r="S3" s="5">
-        <v>8.9198916894983105E-2</v>
+        <v>8.888519016512933E-2</v>
       </c>
       <c r="T3" s="5">
-        <v>1.5985880260153829</v>
+        <v>1.5915908584895087</v>
       </c>
       <c r="U3" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V3" s="5">
-        <v>0.42586190452079686</v>
+        <v>0.43678569903044911</v>
       </c>
       <c r="W3" s="5">
-        <v>2.3589396210390533E-2</v>
+        <v>2.4746642498929054E-2</v>
       </c>
       <c r="X3" s="5">
-        <v>4.0469512525596834</v>
+        <v>4.0522915968346922</v>
       </c>
       <c r="Y3" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z3" s="19">
-        <v>5.7404208881877696E-9</v>
+        <v>1.0218740945602944E-8</v>
       </c>
       <c r="AA3" s="5">
         <f t="shared" ref="AA3:AA17" si="0">R3-A3</f>
-        <v>0.25348612182948604</v>
+        <v>0.26363365135228745</v>
       </c>
       <c r="AB3" s="5">
         <f t="shared" ref="AB3:AB17" si="1">S3-B3</f>
-        <v>-3.0801083105016891E-2</v>
+        <v>-3.1114809834870666E-2</v>
       </c>
       <c r="AC3" s="5">
         <f t="shared" ref="AC3:AC17" si="2">T3-C3</f>
-        <v>2.8588026015382795E-2</v>
+        <v>2.1590858489508591E-2</v>
       </c>
       <c r="AD3" s="5">
         <f t="shared" ref="AD3:AD17" si="3">U3-D3</f>
@@ -2927,15 +2933,15 @@
       </c>
       <c r="AE3" s="5">
         <f t="shared" ref="AE3:AE17" si="4">V3-E3</f>
-        <v>0.12586190452079687</v>
+        <v>0.13678569903044913</v>
       </c>
       <c r="AF3" s="5">
         <f t="shared" ref="AF3:AF17" si="5">W3-F3</f>
-        <v>3.589396210390533E-3</v>
+        <v>4.7466424989290532E-3</v>
       </c>
       <c r="AG3" s="5">
         <f t="shared" ref="AG3:AG17" si="6">X3-G3</f>
-        <v>0.90495125255968345</v>
+        <v>0.9102915968346923</v>
       </c>
       <c r="AH3" s="5">
         <f t="shared" ref="AH3:AH17" si="7">Y3-H3</f>
@@ -2943,15 +2949,15 @@
       </c>
       <c r="AI3" s="9">
         <f>AVERAGE(ABS(AA3),ABS(AE3))</f>
-        <v>0.18967401317514146</v>
+        <v>0.20020967519136829</v>
       </c>
       <c r="AJ3" s="9">
         <f t="shared" ref="AJ3:AK17" si="8">AVERAGE(ABS(AB3),ABS(AF3))</f>
-        <v>1.7195239657703712E-2</v>
+        <v>1.793072616689986E-2</v>
       </c>
       <c r="AK3" s="9">
         <f t="shared" si="8"/>
-        <v>0.46676963928753312</v>
+        <v>0.46594122766210044</v>
       </c>
       <c r="AL3" s="1" t="s">
         <v>23</v>
@@ -3048,43 +3054,43 @@
         <v>-0.190968692302704</v>
       </c>
       <c r="R4" s="14">
-        <v>0.61501210728840638</v>
+        <v>0.2361928483768298</v>
       </c>
       <c r="S4" s="14">
-        <v>7.3854109951049199E-2</v>
+        <v>0.12963296786042683</v>
       </c>
       <c r="T4" s="14">
-        <v>1.6370270376824019</v>
+        <v>1.6532551903303669</v>
       </c>
       <c r="U4" s="14">
         <v>1.5707963267948966</v>
       </c>
       <c r="V4" s="14">
-        <v>0.80438641517548459</v>
+        <v>0.42307346571120047</v>
       </c>
       <c r="W4" s="14">
-        <v>2.8884891143172491E-2</v>
+        <v>2.0000017626560177E-2</v>
       </c>
       <c r="X4" s="14">
-        <v>4.7586045080823576</v>
+        <v>4.7519267340730167</v>
       </c>
       <c r="Y4" s="14">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z4" s="20">
-        <v>1.4900725370779261E-7</v>
+        <v>1.9019607825814942E-7</v>
       </c>
       <c r="AA4" s="14">
         <f t="shared" si="0"/>
-        <v>0.11501210728840638</v>
+        <v>-0.2638071516231702</v>
       </c>
       <c r="AB4" s="14">
         <f t="shared" si="1"/>
-        <v>-4.6145890048950797E-2</v>
+        <v>9.6329678604268332E-3</v>
       </c>
       <c r="AC4" s="14">
         <f t="shared" si="2"/>
-        <v>6.7027037682401813E-2</v>
+        <v>8.3255190330366879E-2</v>
       </c>
       <c r="AD4" s="14">
         <f t="shared" si="3"/>
@@ -3092,15 +3098,15 @@
       </c>
       <c r="AE4" s="14">
         <f t="shared" si="4"/>
-        <v>0.10438641517548464</v>
+        <v>-0.27692653428879949</v>
       </c>
       <c r="AF4" s="14">
         <f t="shared" si="5"/>
-        <v>-3.1115108856827507E-2</v>
+        <v>-3.9999982373439824E-2</v>
       </c>
       <c r="AG4" s="14">
         <f t="shared" si="6"/>
-        <v>4.6604508082357832E-2</v>
+        <v>3.9926734073016945E-2</v>
       </c>
       <c r="AH4" s="14">
         <f t="shared" si="7"/>
@@ -3108,27 +3114,27 @@
       </c>
       <c r="AI4" s="16">
         <f t="shared" ref="AI4:AI17" si="9">AVERAGE(ABS(AA4),ABS(AE4))</f>
-        <v>0.10969926123194551</v>
+        <v>0.27036684295598484</v>
       </c>
       <c r="AJ4" s="16">
         <f t="shared" si="8"/>
-        <v>3.8630499452889155E-2</v>
+        <v>2.4816475116933329E-2</v>
       </c>
       <c r="AK4" s="16">
         <f t="shared" si="8"/>
-        <v>5.6815772882379822E-2</v>
+        <v>6.1590962201691912E-2</v>
       </c>
       <c r="AL4" s="8" cm="1">
         <f t="array" ref="AL4">AVERAGE(ABS(AA3:AA17))</f>
-        <v>0.20415321834156522</v>
+        <v>0.17703122950005459</v>
       </c>
       <c r="AM4" s="8" cm="1">
         <f t="array" ref="AM4">AVERAGE(ABS(AB3:AB17))</f>
-        <v>2.7095625896879045E-2</v>
+        <v>2.042458883533262E-2</v>
       </c>
       <c r="AN4" s="8" cm="1">
         <f t="array" ref="AN4">AVERAGE(ABS(AC3:AC17))</f>
-        <v>0.19243521547032769</v>
+        <v>0.46084094362143507</v>
       </c>
       <c r="AO4" s="8" cm="1">
         <f t="array" ref="AO4">AVERAGE(ABS(AD3:AD17))</f>
@@ -3136,15 +3142,15 @@
       </c>
       <c r="AP4" s="8" cm="1">
         <f t="array" ref="AP4">AVERAGE(ABS(AE3:AE17))</f>
-        <v>0.1248551571503513</v>
+        <v>0.14434075850690156</v>
       </c>
       <c r="AQ4" s="8" cm="1">
         <f t="array" ref="AQ4">AVERAGE(ABS(AF3:AF17))</f>
-        <v>2.4544251932337287E-2</v>
+        <v>2.6830612629143644E-2</v>
       </c>
       <c r="AR4" s="8" cm="1">
         <f t="array" ref="AR4">AVERAGE(ABS(AG3:AG17))</f>
-        <v>0.48429377346619396</v>
+        <v>0.29290432295832597</v>
       </c>
       <c r="AS4" s="8" cm="1">
         <f t="array" ref="AS4">AVERAGE(ABS(AH3:AH17))</f>
@@ -3221,43 +3227,43 @@
         <v>0.28356426954269398</v>
       </c>
       <c r="R5" s="5">
-        <v>0.8019280299229431</v>
+        <v>0.75817542182106845</v>
       </c>
       <c r="S5" s="5">
-        <v>0.17603228319492448</v>
+        <v>0.18070210151059904</v>
       </c>
       <c r="T5" s="5">
-        <v>1.6027352862005662</v>
+        <v>1.6018341710038033</v>
       </c>
       <c r="U5" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V5" s="5">
-        <v>0.35017019559090157</v>
+        <v>0.30463689776690051</v>
       </c>
       <c r="W5" s="5">
-        <v>4.0320914123000137E-2</v>
+        <v>3.2462969578982204E-2</v>
       </c>
       <c r="X5" s="5">
-        <v>4.7766012548779964</v>
+        <v>4.779461427088977</v>
       </c>
       <c r="Y5" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z5" s="19">
-        <v>9.55455386291835E-10</v>
+        <v>2.192318654833206E-7</v>
       </c>
       <c r="AA5" s="5">
         <f t="shared" si="0"/>
-        <v>1.9280299229430531E-3</v>
+        <v>-4.1824578178931593E-2</v>
       </c>
       <c r="AB5" s="5">
         <f t="shared" si="1"/>
-        <v>-3.9677168050755163E-3</v>
+        <v>7.021015105990458E-4</v>
       </c>
       <c r="AC5" s="5">
         <f t="shared" si="2"/>
-        <v>3.2735286200566094E-2</v>
+        <v>3.1834171003803258E-2</v>
       </c>
       <c r="AD5" s="5">
         <f t="shared" si="3"/>
@@ -3265,15 +3271,15 @@
       </c>
       <c r="AE5" s="5">
         <f t="shared" si="4"/>
-        <v>-4.9829804409098455E-2</v>
+        <v>-9.5363102233099517E-2</v>
       </c>
       <c r="AF5" s="5">
         <f t="shared" si="5"/>
-        <v>-3.9679085876999864E-2</v>
+        <v>-4.7537030421017798E-2</v>
       </c>
       <c r="AG5" s="5">
         <f t="shared" si="6"/>
-        <v>6.4601254877996617E-2</v>
+        <v>6.7461427088977288E-2</v>
       </c>
       <c r="AH5" s="5">
         <f t="shared" si="7"/>
@@ -3281,26 +3287,26 @@
       </c>
       <c r="AI5" s="9">
         <f t="shared" si="9"/>
-        <v>2.5878917166020754E-2</v>
+        <v>6.8593840206015555E-2</v>
       </c>
       <c r="AJ5" s="9">
         <f t="shared" si="8"/>
-        <v>2.182340134103769E-2</v>
+        <v>2.4119565965808422E-2</v>
       </c>
       <c r="AK5" s="9">
         <f t="shared" si="8"/>
-        <v>4.8668270539281355E-2</v>
-      </c>
-      <c r="AL5" s="30" t="s">
+        <v>4.9647799046390273E-2</v>
+      </c>
+      <c r="AL5" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="30"/>
-      <c r="AO5" s="30"/>
-      <c r="AP5" s="30"/>
-      <c r="AQ5" s="30"/>
-      <c r="AR5" s="30"/>
-      <c r="AS5" s="30"/>
+      <c r="AM5" s="31"/>
+      <c r="AN5" s="31"/>
+      <c r="AO5" s="31"/>
+      <c r="AP5" s="31"/>
+      <c r="AQ5" s="31"/>
+      <c r="AR5" s="31"/>
+      <c r="AS5" s="31"/>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
@@ -3372,43 +3378,43 @@
         <v>0.13295280933380099</v>
       </c>
       <c r="R6" s="5">
-        <v>0.420466972470177</v>
+        <v>0.52721599036919065</v>
       </c>
       <c r="S6" s="5">
-        <v>0.14460775500964243</v>
+        <v>0.13064266340979669</v>
       </c>
       <c r="T6" s="5">
-        <v>1.8162797445222869</v>
+        <v>1.5692194584815133</v>
       </c>
       <c r="U6" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V6" s="5">
-        <v>0.63046312251809544</v>
+        <v>0.77627959066504493</v>
       </c>
       <c r="W6" s="5">
-        <v>2.7212856945557005E-2</v>
+        <v>4.483867146613775E-2</v>
       </c>
       <c r="X6" s="5">
-        <v>3.5761369619358865</v>
+        <v>3.6594988321543296</v>
       </c>
       <c r="Y6" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z6" s="19">
-        <v>6.6253941111062855E-10</v>
+        <v>6.96360561720752E-8</v>
       </c>
       <c r="AA6" s="5">
         <f t="shared" si="0"/>
-        <v>0.12046697247017701</v>
+        <v>0.22721599036919066</v>
       </c>
       <c r="AB6" s="5">
         <f t="shared" si="1"/>
-        <v>-5.5392244990357581E-2</v>
+        <v>-6.9357336590203322E-2</v>
       </c>
       <c r="AC6" s="5">
         <f t="shared" si="2"/>
-        <v>0.24627974452228685</v>
+        <v>-7.8054151848672149E-4</v>
       </c>
       <c r="AD6" s="5">
         <f t="shared" si="3"/>
@@ -3416,15 +3422,15 @@
       </c>
       <c r="AE6" s="5">
         <f t="shared" si="4"/>
-        <v>-6.9536877481904513E-2</v>
+        <v>7.6279590665044972E-2</v>
       </c>
       <c r="AF6" s="5">
         <f t="shared" si="5"/>
-        <v>-1.2787143054442996E-2</v>
+        <v>4.8386714661377492E-3</v>
       </c>
       <c r="AG6" s="5">
         <f t="shared" si="6"/>
-        <v>0.43413696193588658</v>
+        <v>0.51749883215432968</v>
       </c>
       <c r="AH6" s="5">
         <f t="shared" si="7"/>
@@ -3432,15 +3438,15 @@
       </c>
       <c r="AI6" s="9">
         <f t="shared" si="9"/>
-        <v>9.5001924976040764E-2</v>
+        <v>0.15174779051711781</v>
       </c>
       <c r="AJ6" s="9">
         <f t="shared" si="8"/>
-        <v>3.4089694022400287E-2</v>
+        <v>3.7098004028170539E-2</v>
       </c>
       <c r="AK6" s="9">
         <f t="shared" si="8"/>
-        <v>0.34020835322908671</v>
+        <v>0.2591396868364082</v>
       </c>
       <c r="AL6" s="7" t="s">
         <v>33</v>
@@ -3527,43 +3533,43 @@
         <v>-0.48219949007034302</v>
       </c>
       <c r="R7" s="5">
-        <v>0.60707540853132202</v>
+        <v>0.60713301008119613</v>
       </c>
       <c r="S7" s="5">
-        <v>9.1008946053146314E-2</v>
+        <v>9.0858055647504404E-2</v>
       </c>
       <c r="T7" s="5">
-        <v>2.9864978806336673</v>
+        <v>2.9813250275329457</v>
       </c>
       <c r="U7" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V7" s="5">
-        <v>0.66197406831519079</v>
+        <v>0.66459208617919552</v>
       </c>
       <c r="W7" s="5">
-        <v>8.6409605139190701E-2</v>
+        <v>8.6605784603893468E-2</v>
       </c>
       <c r="X7" s="5">
-        <v>4.2357289252120864</v>
+        <v>4.2368231284953302</v>
       </c>
       <c r="Y7" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z7" s="19">
-        <v>5.2607573499500193E-6</v>
+        <v>2.7453203073212905E-6</v>
       </c>
       <c r="AA7" s="5">
         <f t="shared" si="0"/>
-        <v>0.30707540853132204</v>
+        <v>0.30713301008119614</v>
       </c>
       <c r="AB7" s="5">
         <f t="shared" si="1"/>
-        <v>-8.9910539468536915E-3</v>
+        <v>-9.1419443524956012E-3</v>
       </c>
       <c r="AC7" s="5">
         <f t="shared" si="2"/>
-        <v>-0.15550211936633263</v>
+        <v>-0.1606749724670542</v>
       </c>
       <c r="AD7" s="5">
         <f t="shared" si="3"/>
@@ -3571,15 +3577,15 @@
       </c>
       <c r="AE7" s="5">
         <f t="shared" si="4"/>
-        <v>-0.13802593168480926</v>
+        <v>-0.13540791382080453</v>
       </c>
       <c r="AF7" s="5">
         <f t="shared" si="5"/>
-        <v>6.4096051391906994E-3</v>
+        <v>6.6057846038934664E-3</v>
       </c>
       <c r="AG7" s="5">
         <f t="shared" si="6"/>
-        <v>0.30872892521208639</v>
+        <v>0.30982312849533011</v>
       </c>
       <c r="AH7" s="5">
         <f t="shared" si="7"/>
@@ -3587,27 +3593,27 @@
       </c>
       <c r="AI7" s="9">
         <f t="shared" si="9"/>
-        <v>0.22255067010806565</v>
+        <v>0.22127046195100034</v>
       </c>
       <c r="AJ7" s="9">
         <f t="shared" si="8"/>
-        <v>7.7003295430221955E-3</v>
+        <v>7.8738644781945338E-3</v>
       </c>
       <c r="AK7" s="9">
         <f t="shared" si="8"/>
-        <v>0.23211552228920951</v>
+        <v>0.23524905048119216</v>
       </c>
       <c r="AL7" s="11">
         <f>AVERAGE(AL4,AP4)</f>
-        <v>0.16450418774595826</v>
+        <v>0.16068599400347808</v>
       </c>
       <c r="AM7" s="11">
         <f t="shared" ref="AM7:AN7" si="10">AVERAGE(AM4,AQ4)</f>
-        <v>2.5819938914608168E-2</v>
+        <v>2.362760073223813E-2</v>
       </c>
       <c r="AN7" s="11">
         <f t="shared" si="10"/>
-        <v>0.33836449446826083</v>
+        <v>0.37687263328988052</v>
       </c>
       <c r="AO7" s="8"/>
       <c r="AP7" s="8"/>
@@ -3685,43 +3691,43 @@
         <v>-0.22229230403900099</v>
       </c>
       <c r="R8" s="5">
-        <v>0.15312984346615566</v>
+        <v>0.8144252781731437</v>
       </c>
       <c r="S8" s="5">
-        <v>0.158812840670088</v>
+        <v>9.6125258969866748E-2</v>
       </c>
       <c r="T8" s="5">
-        <v>2.6353326541999564</v>
+        <v>2.8815087289782082</v>
       </c>
       <c r="U8" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V8" s="5">
-        <v>0.99998512033524956</v>
+        <v>0.52750015746723689</v>
       </c>
       <c r="W8" s="5">
-        <v>8.0562070070799754E-2</v>
+        <v>7.4228373720110985E-2</v>
       </c>
       <c r="X8" s="5">
-        <v>3.4427387429561418</v>
+        <v>4.1023158331038303</v>
       </c>
       <c r="Y8" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z8" s="19">
-        <v>1.9521376173681426E-7</v>
+        <v>3.7668415371455878E-7</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="0"/>
-        <v>-0.5468701565338443</v>
+        <v>0.11442527817314374</v>
       </c>
       <c r="AB8" s="5">
         <f t="shared" si="1"/>
-        <v>5.881284067008799E-2</v>
+        <v>-3.874741030133258E-3</v>
       </c>
       <c r="AC8" s="5">
         <f t="shared" si="2"/>
-        <v>-0.50666734580004347</v>
+        <v>-0.2604912710217917</v>
       </c>
       <c r="AD8" s="5">
         <f t="shared" si="3"/>
@@ -3729,15 +3735,15 @@
       </c>
       <c r="AE8" s="5">
         <f t="shared" si="4"/>
-        <v>0.59998512033524953</v>
+        <v>0.12750015746723686</v>
       </c>
       <c r="AF8" s="5">
         <f t="shared" si="5"/>
-        <v>4.0562070070799754E-2</v>
+        <v>3.4228373720110984E-2</v>
       </c>
       <c r="AG8" s="5">
         <f t="shared" si="6"/>
-        <v>-0.48426125704385825</v>
+        <v>0.17531583310383025</v>
       </c>
       <c r="AH8" s="5">
         <f t="shared" si="7"/>
@@ -3745,15 +3751,15 @@
       </c>
       <c r="AI8" s="10">
         <f t="shared" si="9"/>
-        <v>0.57342763843454692</v>
+        <v>0.1209627178201903</v>
       </c>
       <c r="AJ8" s="10">
         <f t="shared" si="8"/>
-        <v>4.9687455370443875E-2</v>
+        <v>1.9051557375122121E-2</v>
       </c>
       <c r="AK8" s="10">
         <f t="shared" si="8"/>
-        <v>0.49546430142195086</v>
+        <v>0.21790355206281098</v>
       </c>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.25">
@@ -3826,43 +3832,43 @@
         <v>-0.380674779415131</v>
       </c>
       <c r="R9" s="5">
-        <v>0.59153808171597488</v>
+        <v>0.64637441469415347</v>
       </c>
       <c r="S9" s="5">
-        <v>0.13314790650593747</v>
+        <v>0.12953535920944981</v>
       </c>
       <c r="T9" s="5">
-        <v>2.9154405279629465</v>
+        <v>2.8837153646999623</v>
       </c>
       <c r="U9" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V9" s="5">
-        <v>0.68888684753855101</v>
+        <v>0.68389247067324233</v>
       </c>
       <c r="W9" s="5">
-        <v>0.10293202867129436</v>
+        <v>0.1043476293615514</v>
       </c>
       <c r="X9" s="5">
-        <v>4.0087739037391907</v>
+        <v>4.0916041799748522</v>
       </c>
       <c r="Y9" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z9" s="19">
-        <v>1.0436398774810899E-8</v>
+        <v>9.2540084858739116E-7</v>
       </c>
       <c r="AA9" s="5">
         <f t="shared" si="0"/>
-        <v>9.1538081715974884E-2</v>
+        <v>0.14637441469415347</v>
       </c>
       <c r="AB9" s="5">
         <f t="shared" si="1"/>
-        <v>-6.8520934940625444E-3</v>
+        <v>-1.0464640790550206E-2</v>
       </c>
       <c r="AC9" s="5">
         <f t="shared" si="2"/>
-        <v>-0.2265594720370534</v>
+        <v>-0.25828463530003765</v>
       </c>
       <c r="AD9" s="5">
         <f t="shared" si="3"/>
@@ -3870,15 +3876,15 @@
       </c>
       <c r="AE9" s="5">
         <f t="shared" si="4"/>
-        <v>-1.111315246144895E-2</v>
+        <v>-1.610752932675763E-2</v>
       </c>
       <c r="AF9" s="5">
         <f t="shared" si="5"/>
-        <v>2.2932028671294361E-2</v>
+        <v>2.4347629361551396E-2</v>
       </c>
       <c r="AG9" s="5">
         <f t="shared" si="6"/>
-        <v>8.177390373919069E-2</v>
+        <v>0.16460417997485211</v>
       </c>
       <c r="AH9" s="5">
         <f t="shared" si="7"/>
@@ -3886,15 +3892,15 @@
       </c>
       <c r="AI9" s="9">
         <f t="shared" si="9"/>
-        <v>5.1325617088711917E-2</v>
+        <v>8.1240972010455548E-2</v>
       </c>
       <c r="AJ9" s="9">
         <f t="shared" si="8"/>
-        <v>1.4892061082678452E-2</v>
+        <v>1.7406135076050801E-2</v>
       </c>
       <c r="AK9" s="9">
         <f t="shared" si="8"/>
-        <v>0.15416668788812204</v>
+        <v>0.21144440763744488</v>
       </c>
       <c r="AL9" s="13"/>
       <c r="AM9" s="13"/>
@@ -3970,43 +3976,43 @@
         <v>-0.296476870775223</v>
       </c>
       <c r="R10" s="5">
-        <v>0.77150886662211471</v>
+        <v>0.77057969060101694</v>
       </c>
       <c r="S10" s="5">
-        <v>0.13141799449895897</v>
+        <v>0.13106213675642675</v>
       </c>
       <c r="T10" s="5">
-        <v>2.8261691241517952</v>
+        <v>2.8258416527406154</v>
       </c>
       <c r="U10" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V10" s="5">
-        <v>0.63741601380028268</v>
+        <v>0.63701334027023304</v>
       </c>
       <c r="W10" s="5">
-        <v>9.9296152032712609E-2</v>
+        <v>9.9807208834126471E-2</v>
       </c>
       <c r="X10" s="5">
-        <v>4.1544849611370465</v>
+        <v>4.1514962125184747</v>
       </c>
       <c r="Y10" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z10" s="19">
-        <v>3.8361133017192555E-7</v>
+        <v>9.7908619354922661E-7</v>
       </c>
       <c r="AA10" s="5">
         <f t="shared" si="0"/>
-        <v>7.1508866622114753E-2</v>
+        <v>7.0579690601016987E-2</v>
       </c>
       <c r="AB10" s="5">
         <f t="shared" si="1"/>
-        <v>-8.5820055010410456E-3</v>
+        <v>-8.937863243573263E-3</v>
       </c>
       <c r="AC10" s="5">
         <f t="shared" si="2"/>
-        <v>-0.31583087584820468</v>
+        <v>-0.31615834725938452</v>
       </c>
       <c r="AD10" s="5">
         <f t="shared" si="3"/>
@@ -4014,15 +4020,15 @@
       </c>
       <c r="AE10" s="5">
         <f t="shared" si="4"/>
-        <v>0.13741601380028268</v>
+        <v>0.13701334027023304</v>
       </c>
       <c r="AF10" s="5">
         <f t="shared" si="5"/>
-        <v>3.9296152032712611E-2</v>
+        <v>3.9807208834126473E-2</v>
       </c>
       <c r="AG10" s="5">
         <f t="shared" si="6"/>
-        <v>0.22748496113704642</v>
+        <v>0.22449621251847462</v>
       </c>
       <c r="AH10" s="5">
         <f t="shared" si="7"/>
@@ -4030,15 +4036,15 @@
       </c>
       <c r="AI10" s="9">
         <f t="shared" si="9"/>
-        <v>0.10446244021119871</v>
+        <v>0.10379651543562501</v>
       </c>
       <c r="AJ10" s="9">
         <f t="shared" si="8"/>
-        <v>2.3939078766876828E-2</v>
+        <v>2.4372536038849868E-2</v>
       </c>
       <c r="AK10" s="9">
         <f t="shared" si="8"/>
-        <v>0.27165791849262555</v>
+        <v>0.27032727988892957</v>
       </c>
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.25">
@@ -4111,43 +4117,43 @@
         <v>-0.23403739929199199</v>
       </c>
       <c r="R11" s="5">
-        <v>0.2641148139595752</v>
+        <v>0.26678114285968224</v>
       </c>
       <c r="S11" s="5">
-        <v>0.18202031217043588</v>
+        <v>0.18110205090970105</v>
       </c>
       <c r="T11" s="5">
-        <v>2.4192451452119119</v>
+        <v>2.4156391455236372</v>
       </c>
       <c r="U11" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V11" s="5">
-        <v>0.59373935599664018</v>
+        <v>0.5941161585705077</v>
       </c>
       <c r="W11" s="5">
-        <v>9.3598741733366173E-2</v>
+        <v>9.3832982205083446E-2</v>
       </c>
       <c r="X11" s="5">
-        <v>3.8958881173858528</v>
+        <v>3.9005298078518709</v>
       </c>
       <c r="Y11" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z11" s="19">
-        <v>5.2798407825688896E-9</v>
+        <v>6.1997032788828846E-7</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="0"/>
-        <v>-0.13588518604042482</v>
+        <v>-0.13321885714031778</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="1"/>
-        <v>2.020312170435884E-3</v>
+        <v>1.1020509097010578E-3</v>
       </c>
       <c r="AC11" s="5">
         <f t="shared" si="2"/>
-        <v>-0.72275485478808799</v>
+        <v>-0.72636085447636267</v>
       </c>
       <c r="AD11" s="5">
         <f t="shared" si="3"/>
@@ -4155,15 +4161,15 @@
       </c>
       <c r="AE11" s="5">
         <f t="shared" si="4"/>
-        <v>0.19373935599664016</v>
+        <v>0.19411615857050768</v>
       </c>
       <c r="AF11" s="5">
         <f t="shared" si="5"/>
-        <v>7.3598741733366169E-2</v>
+        <v>7.3832982205083442E-2</v>
       </c>
       <c r="AG11" s="5">
         <f t="shared" si="6"/>
-        <v>-3.1111882614147213E-2</v>
+        <v>-2.6470192148129179E-2</v>
       </c>
       <c r="AH11" s="5">
         <f t="shared" si="7"/>
@@ -4171,15 +4177,15 @@
       </c>
       <c r="AI11" s="9">
         <f t="shared" si="9"/>
-        <v>0.16481227101853249</v>
+        <v>0.16366750785541273</v>
       </c>
       <c r="AJ11" s="9">
         <f t="shared" si="8"/>
-        <v>3.7809526951901026E-2</v>
+        <v>3.746751655739225E-2</v>
       </c>
       <c r="AK11" s="9">
         <f t="shared" si="8"/>
-        <v>0.3769333687011176</v>
+        <v>0.37641552331224593</v>
       </c>
       <c r="AL11" s="13"/>
       <c r="AM11" s="13"/>
@@ -4255,43 +4261,43 @@
         <v>-0.46333062648773199</v>
       </c>
       <c r="R12" s="5">
-        <v>0.74443735012885348</v>
+        <v>0.97831711335596638</v>
       </c>
       <c r="S12" s="5">
-        <v>0.16739676127741501</v>
+        <v>0.15277152791140047</v>
       </c>
       <c r="T12" s="5">
-        <v>2.905499374475716</v>
+        <v>3.0942799368390244</v>
       </c>
       <c r="U12" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V12" s="5">
-        <v>0.86835712261845432</v>
+        <v>0.60983392468265252</v>
       </c>
       <c r="W12" s="5">
-        <v>8.2162012403960274E-2</v>
+        <v>6.0676688669076488E-2</v>
       </c>
       <c r="X12" s="5">
-        <v>3.9663755649672563</v>
+        <v>4.1349589044002881</v>
       </c>
       <c r="Y12" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z12" s="19">
-        <v>1.735818570121724E-7</v>
+        <v>1.4352086796852891E-6</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="0"/>
-        <v>4.4437350128853526E-2</v>
+        <v>0.27831711335596643</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="1"/>
-        <v>-1.2603238722584981E-2</v>
+        <v>-2.722847208859952E-2</v>
       </c>
       <c r="AC12" s="5">
         <f t="shared" si="2"/>
-        <v>-0.23650062552428386</v>
+        <v>-4.7720063160975545E-2</v>
       </c>
       <c r="AD12" s="5">
         <f t="shared" si="3"/>
@@ -4299,15 +4305,15 @@
       </c>
       <c r="AE12" s="5">
         <f t="shared" si="4"/>
-        <v>6.835712261845428E-2</v>
+        <v>-0.19016607531734753</v>
       </c>
       <c r="AF12" s="5">
         <f t="shared" si="5"/>
-        <v>4.2162012403960274E-2</v>
+        <v>2.0676688669076487E-2</v>
       </c>
       <c r="AG12" s="5">
         <f t="shared" si="6"/>
-        <v>3.9375564967256249E-2</v>
+        <v>0.20795890440028808</v>
       </c>
       <c r="AH12" s="5">
         <f t="shared" si="7"/>
@@ -4315,15 +4321,15 @@
       </c>
       <c r="AI12" s="9">
         <f t="shared" si="9"/>
-        <v>5.6397236373653903E-2</v>
+        <v>0.23424159433665698</v>
       </c>
       <c r="AJ12" s="9">
         <f t="shared" si="8"/>
-        <v>2.7382625563272627E-2</v>
+        <v>2.3952580378838004E-2</v>
       </c>
       <c r="AK12" s="9">
         <f t="shared" si="8"/>
-        <v>0.13793809524577005</v>
+        <v>0.12783948378063181</v>
       </c>
     </row>
     <row r="13" spans="1:45" x14ac:dyDescent="0.25">
@@ -4396,43 +4402,43 @@
         <v>-0.59106355905532804</v>
       </c>
       <c r="R13" s="5">
-        <v>0.85056815635664629</v>
+        <v>0.17620896176457868</v>
       </c>
       <c r="S13" s="5">
-        <v>7.7557827187846623E-2</v>
+        <v>9.9286257032007066E-2</v>
       </c>
       <c r="T13" s="5">
-        <v>4.7205624614308261</v>
+        <v>0.12186637325268596</v>
       </c>
       <c r="U13" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V13" s="5">
-        <v>0.26360679350106492</v>
+        <v>0.65619757764419362</v>
       </c>
       <c r="W13" s="5">
-        <v>5.4148218840250145E-2</v>
+        <v>8.8113330033240705E-2</v>
       </c>
       <c r="X13" s="5">
-        <v>1.8021127564263479</v>
+        <v>4.3571793173094253</v>
       </c>
       <c r="Y13" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z13" s="19">
-        <v>3.7672500991470073E-8</v>
+        <v>8.7905820271715823E-8</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="0"/>
-        <v>0.55056815635664624</v>
+        <v>-0.12379103823542131</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="1"/>
-        <v>-4.2442172812153373E-2</v>
+        <v>-2.0713742967992929E-2</v>
       </c>
       <c r="AC13" s="5">
         <f t="shared" si="2"/>
-        <v>8.5624614308263958E-3</v>
+        <v>-4.5901336267473134</v>
       </c>
       <c r="AD13" s="5">
         <f t="shared" si="3"/>
@@ -4440,15 +4446,15 @@
       </c>
       <c r="AE13" s="5">
         <f t="shared" si="4"/>
-        <v>-3.6393206498935071E-2</v>
+        <v>0.35619757764419363</v>
       </c>
       <c r="AF13" s="5">
         <f t="shared" si="5"/>
-        <v>1.4148218840250144E-2</v>
+        <v>4.8113330033240705E-2</v>
       </c>
       <c r="AG13" s="5">
         <f t="shared" si="6"/>
-        <v>-2.9098872435736518</v>
+        <v>-0.35482068269057443</v>
       </c>
       <c r="AH13" s="5">
         <f t="shared" si="7"/>
@@ -4456,15 +4462,15 @@
       </c>
       <c r="AI13" s="9">
         <f t="shared" si="9"/>
-        <v>0.29348068142779066</v>
+        <v>0.23999430793980747</v>
       </c>
       <c r="AJ13" s="9">
         <f t="shared" si="8"/>
-        <v>2.8295195826201758E-2</v>
+        <v>3.441353650061682E-2</v>
       </c>
       <c r="AK13" s="9">
         <f t="shared" si="8"/>
-        <v>1.4592248525022391</v>
+        <v>2.4724771547189439</v>
       </c>
       <c r="AL13" s="13"/>
       <c r="AM13" s="13"/>
@@ -4540,43 +4546,43 @@
         <v>-0.86990654468536399</v>
       </c>
       <c r="R14" s="5">
-        <v>0.96313294184985332</v>
+        <v>0.95728856181666944</v>
       </c>
       <c r="S14" s="5">
-        <v>0.11573459996829016</v>
+        <v>0.11629478017871611</v>
       </c>
       <c r="T14" s="5">
-        <v>4.67188229418998</v>
+        <v>4.6704620216669444</v>
       </c>
       <c r="U14" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V14" s="5">
-        <v>0.66503572447894166</v>
+        <v>0.66378324995961235</v>
       </c>
       <c r="W14" s="5">
-        <v>2.0203519249011218E-2</v>
+        <v>2.0010429330519604E-2</v>
       </c>
       <c r="X14" s="5">
-        <v>3.0673489601123038</v>
+        <v>3.0768212349740671</v>
       </c>
       <c r="Y14" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z14" s="19">
-        <v>5.8574947019272704E-7</v>
+        <v>4.2614175506698193E-7</v>
       </c>
       <c r="AA14" s="5">
         <f t="shared" si="0"/>
-        <v>0.16313294184985327</v>
+        <v>0.15728856181666939</v>
       </c>
       <c r="AB14" s="5">
         <f t="shared" si="1"/>
-        <v>-4.2654000317098317E-3</v>
+        <v>-3.7052198212838838E-3</v>
       </c>
       <c r="AC14" s="5">
         <f t="shared" si="2"/>
-        <v>-4.0117705810019721E-2</v>
+        <v>-4.1537978333055392E-2</v>
       </c>
       <c r="AD14" s="5">
         <f t="shared" si="3"/>
@@ -4584,15 +4590,15 @@
       </c>
       <c r="AE14" s="5">
         <f t="shared" si="4"/>
-        <v>-3.4964275521058297E-2</v>
+        <v>-3.6216750040387602E-2</v>
       </c>
       <c r="AF14" s="5">
         <f t="shared" si="5"/>
-        <v>2.0351924901121712E-4</v>
+        <v>1.0429330519604041E-5</v>
       </c>
       <c r="AG14" s="5">
         <f t="shared" si="6"/>
-        <v>-7.4651039887696058E-2</v>
+        <v>-6.5178765025932783E-2</v>
       </c>
       <c r="AH14" s="5">
         <f t="shared" si="7"/>
@@ -4600,15 +4606,15 @@
       </c>
       <c r="AI14" s="9">
         <f t="shared" si="9"/>
-        <v>9.9048608685455786E-2</v>
+        <v>9.6752655928528497E-2</v>
       </c>
       <c r="AJ14" s="9">
         <f t="shared" si="8"/>
-        <v>2.2344596403605244E-3</v>
+        <v>1.8578245759017439E-3</v>
       </c>
       <c r="AK14" s="9">
         <f t="shared" si="8"/>
-        <v>5.738437284885789E-2</v>
+        <v>5.3358371679494088E-2</v>
       </c>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.25">
@@ -4681,43 +4687,43 @@
         <v>-0.37272521853446999</v>
       </c>
       <c r="R15" s="5">
-        <v>0.79908970812182323</v>
+        <v>0.69971262479204777</v>
       </c>
       <c r="S15" s="5">
-        <v>0.10679225625647949</v>
+        <v>0.11556320577332801</v>
       </c>
       <c r="T15" s="5">
-        <v>4.463986983253486</v>
+        <v>4.415148212454814</v>
       </c>
       <c r="U15" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V15" s="5">
-        <v>0.49357078732614001</v>
+        <v>0.40924275139356486</v>
       </c>
       <c r="W15" s="5">
-        <v>2.9187507496642305E-2</v>
+        <v>2.0993314529002112E-2</v>
       </c>
       <c r="X15" s="5">
-        <v>2.2319726513904712</v>
+        <v>2.3753136829666475</v>
       </c>
       <c r="Y15" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z15" s="19">
-        <v>3.0441949527082943E-8</v>
+        <v>3.8088550880511999E-7</v>
       </c>
       <c r="AA15" s="5">
         <f t="shared" si="0"/>
-        <v>0.39908970812182321</v>
+        <v>0.29971262479204774</v>
       </c>
       <c r="AB15" s="5">
         <f t="shared" si="1"/>
-        <v>-7.3207743743520501E-2</v>
+        <v>-6.4436794226671978E-2</v>
       </c>
       <c r="AC15" s="5">
         <f t="shared" si="2"/>
-        <v>-0.24801301674651377</v>
+        <v>-0.29685178754518571</v>
       </c>
       <c r="AD15" s="5">
         <f t="shared" si="3"/>
@@ -4725,15 +4731,15 @@
       </c>
       <c r="AE15" s="5">
         <f t="shared" si="4"/>
-        <v>-6.4292126738599853E-3</v>
+        <v>-9.0757248606435137E-2</v>
       </c>
       <c r="AF15" s="5">
         <f t="shared" si="5"/>
-        <v>-3.0812492503357693E-2</v>
+        <v>-3.9006685470997886E-2</v>
       </c>
       <c r="AG15" s="5">
         <f t="shared" si="6"/>
-        <v>-0.91002734860952872</v>
+        <v>-0.76668631703335244</v>
       </c>
       <c r="AH15" s="5">
         <f t="shared" si="7"/>
@@ -4741,15 +4747,15 @@
       </c>
       <c r="AI15" s="9">
         <f t="shared" si="9"/>
-        <v>0.2027594603978416</v>
+        <v>0.19523493669924144</v>
       </c>
       <c r="AJ15" s="9">
         <f t="shared" si="8"/>
-        <v>5.20101181234391E-2</v>
+        <v>5.1721739848834936E-2</v>
       </c>
       <c r="AK15" s="9">
         <f t="shared" si="8"/>
-        <v>0.57902018267802124</v>
+        <v>0.53176905228926907</v>
       </c>
     </row>
     <row r="16" spans="1:45" x14ac:dyDescent="0.25">
@@ -4822,43 +4828,43 @@
         <v>-1.05074739456177</v>
       </c>
       <c r="R16" s="5">
-        <v>0.61153017761496586</v>
+        <v>0.62762904706019684</v>
       </c>
       <c r="S16" s="5">
-        <v>0.15908244702698321</v>
+        <v>0.15592001226964788</v>
       </c>
       <c r="T16" s="5">
-        <v>4.6633997241134617</v>
+        <v>4.6658380803727662</v>
       </c>
       <c r="U16" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V16" s="5">
-        <v>0.45827334574417955</v>
+        <v>0.44377945999398916</v>
       </c>
       <c r="W16" s="5">
-        <v>2.0000000002754374E-2</v>
+        <v>2.0084377410258255E-2</v>
       </c>
       <c r="X16" s="5">
-        <v>4.6784400757844065</v>
+        <v>4.674487308102333</v>
       </c>
       <c r="Y16" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z16" s="19">
-        <v>1.3411288788974802E-6</v>
+        <v>2.9722812632829164E-6</v>
       </c>
       <c r="AA16" s="5">
         <f t="shared" si="0"/>
-        <v>0.11153017761496586</v>
+        <v>0.12762904706019684</v>
       </c>
       <c r="AB16" s="5">
         <f t="shared" si="1"/>
-        <v>-4.0917552973016802E-2</v>
+        <v>-4.4079987730352127E-2</v>
       </c>
       <c r="AC16" s="5">
         <f t="shared" si="2"/>
-        <v>-4.8600275886538036E-2</v>
+        <v>-4.6161919627233594E-2</v>
       </c>
       <c r="AD16" s="5">
         <f t="shared" si="3"/>
@@ -4866,15 +4872,15 @@
       </c>
       <c r="AE16" s="5">
         <f t="shared" si="4"/>
-        <v>-0.24172665425582041</v>
+        <v>-0.2562205400060108</v>
       </c>
       <c r="AF16" s="5">
         <f t="shared" si="5"/>
-        <v>2.7543731184742626E-12</v>
+        <v>8.4377410258254515E-5</v>
       </c>
       <c r="AG16" s="5">
         <f t="shared" si="6"/>
-        <v>-3.3559924215593284E-2</v>
+        <v>-3.7512691897666706E-2</v>
       </c>
       <c r="AH16" s="5">
         <f t="shared" si="7"/>
@@ -4882,15 +4888,15 @@
       </c>
       <c r="AI16" s="9">
         <f t="shared" si="9"/>
-        <v>0.17662841593539313</v>
+        <v>0.19192479353310382</v>
       </c>
       <c r="AJ16" s="9">
         <f t="shared" si="8"/>
-        <v>2.0458776487885588E-2</v>
+        <v>2.2082182570305191E-2</v>
       </c>
       <c r="AK16" s="9">
         <f t="shared" si="8"/>
-        <v>4.108010005106566E-2</v>
+        <v>4.183730576245015E-2</v>
       </c>
     </row>
     <row r="17" spans="1:37" x14ac:dyDescent="0.25">
@@ -4963,43 +4969,43 @@
         <v>-0.37296327948570301</v>
       </c>
       <c r="R17" s="5">
-        <v>0.84976901009664274</v>
+        <v>0.80051743502710881</v>
       </c>
       <c r="S17" s="5">
-        <v>0.18856696056168176</v>
+        <v>0.19812384042746445</v>
       </c>
       <c r="T17" s="5">
-        <v>4.7092106156036255</v>
+        <v>4.742777937040966</v>
       </c>
       <c r="U17" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V17" s="5">
-        <v>0.35506230982142589</v>
+        <v>0.34005316031621635</v>
       </c>
       <c r="W17" s="5">
-        <v>9.0868204339701164E-2</v>
+        <v>9.8623373038771583E-2</v>
       </c>
       <c r="X17" s="5">
-        <v>2.4287494264630705</v>
+        <v>2.6164806530645572</v>
       </c>
       <c r="Y17" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z17" s="19">
-        <v>4.6937917074889984E-8</v>
+        <v>2.1845103513639877E-7</v>
       </c>
       <c r="AA17" s="5">
         <f t="shared" si="0"/>
-        <v>0.14976901009664279</v>
+        <v>0.10051743502710886</v>
       </c>
       <c r="AB17" s="5">
         <f t="shared" si="1"/>
-        <v>-1.1433039438318249E-2</v>
+        <v>-1.8761595725355629E-3</v>
       </c>
       <c r="AC17" s="5">
         <f t="shared" si="2"/>
-        <v>-2.7893843963742171E-3</v>
+        <v>3.0777937040966208E-2</v>
       </c>
       <c r="AD17" s="5">
         <f t="shared" si="3"/>
@@ -5007,15 +5013,15 @@
       </c>
       <c r="AE17" s="5">
         <f t="shared" si="4"/>
-        <v>5.5062309821425903E-2</v>
+        <v>4.0053160316216363E-2</v>
       </c>
       <c r="AF17" s="5">
         <f t="shared" si="5"/>
-        <v>1.0868204339701162E-2</v>
+        <v>1.8623373038771582E-2</v>
       </c>
       <c r="AG17" s="5">
         <f t="shared" si="6"/>
-        <v>-0.71325057353692944</v>
+        <v>-0.52551934693544267</v>
       </c>
       <c r="AH17" s="5">
         <f t="shared" si="7"/>
@@ -5023,15 +5029,15 @@
       </c>
       <c r="AI17" s="9">
         <f t="shared" si="9"/>
-        <v>0.10241565995903434</v>
+        <v>7.0285297671662611E-2</v>
       </c>
       <c r="AJ17" s="9">
         <f t="shared" si="8"/>
-        <v>1.1150621889009706E-2</v>
+        <v>1.0249766305653572E-2</v>
       </c>
       <c r="AK17" s="9">
         <f t="shared" si="8"/>
-        <v>0.35801997896665183</v>
+        <v>0.27814864198820444</v>
       </c>
     </row>
   </sheetData>
@@ -5090,61 +5096,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="23" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="33" t="s">
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="S1" s="34"/>
-      <c r="T1" s="34"/>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
-      <c r="W1" s="34"/>
-      <c r="X1" s="34"/>
-      <c r="Y1" s="34"/>
-      <c r="Z1" s="34"/>
-      <c r="AA1" s="31" t="s">
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="35"/>
+      <c r="Y1" s="35"/>
+      <c r="Z1" s="35"/>
+      <c r="AA1" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-      <c r="AF1" s="31"/>
-      <c r="AG1" s="31"/>
-      <c r="AH1" s="31"/>
-      <c r="AI1" s="32" t="s">
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="32"/>
+      <c r="AD1" s="32"/>
+      <c r="AE1" s="32"/>
+      <c r="AF1" s="32"/>
+      <c r="AG1" s="32"/>
+      <c r="AH1" s="32"/>
+      <c r="AI1" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="AJ1" s="32"/>
-      <c r="AK1" s="32"/>
-      <c r="AL1" s="32"/>
-      <c r="AM1" s="32"/>
-      <c r="AN1" s="32"/>
-      <c r="AO1" s="32"/>
-      <c r="AP1" s="32"/>
-      <c r="AQ1" s="32"/>
-      <c r="AR1" s="32"/>
-      <c r="AS1" s="32"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="33"/>
+      <c r="AR1" s="33"/>
+      <c r="AS1" s="33"/>
     </row>
     <row r="2" spans="1:45" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -5258,16 +5264,16 @@
       <c r="AK2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="AL2" s="30" t="s">
+      <c r="AL2" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AM2" s="30"/>
-      <c r="AN2" s="30"/>
-      <c r="AO2" s="30"/>
-      <c r="AP2" s="30"/>
-      <c r="AQ2" s="30"/>
-      <c r="AR2" s="30"/>
-      <c r="AS2" s="30"/>
+      <c r="AM2" s="31"/>
+      <c r="AN2" s="31"/>
+      <c r="AO2" s="31"/>
+      <c r="AP2" s="31"/>
+      <c r="AQ2" s="31"/>
+      <c r="AR2" s="31"/>
+      <c r="AS2" s="31"/>
     </row>
     <row r="3" spans="1:45" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
@@ -5339,43 +5345,43 @@
         <v>0.41270199418067899</v>
       </c>
       <c r="R3" s="5">
-        <v>0.46494919406425178</v>
+        <v>0.66837675427215204</v>
       </c>
       <c r="S3" s="5">
-        <v>0.12939584928923337</v>
+        <v>0.10849019352330234</v>
       </c>
       <c r="T3" s="5">
-        <v>1.6190715077517868</v>
+        <v>1.417559393913534</v>
       </c>
       <c r="U3" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V3" s="5">
-        <v>0.26409831164704506</v>
+        <v>0.45189914217674876</v>
       </c>
       <c r="W3" s="5">
-        <v>2.0009487707417728E-2</v>
+        <v>5.0591238866007679E-2</v>
       </c>
       <c r="X3" s="5">
-        <v>3.3050218707657288</v>
+        <v>3.7018615783648046</v>
       </c>
       <c r="Y3" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z3" s="12">
-        <v>5.5579083927524182E-6</v>
+        <v>3.3190752053599939E-6</v>
       </c>
       <c r="AA3" s="5">
         <f t="shared" ref="AA3:AH17" si="0">R3-A3</f>
-        <v>-3.5050805935748219E-2</v>
+        <v>0.16837675427215204</v>
       </c>
       <c r="AB3" s="5">
         <f t="shared" si="0"/>
-        <v>9.3958492892333711E-3</v>
+        <v>-1.1509806476697651E-2</v>
       </c>
       <c r="AC3" s="5">
         <f t="shared" si="0"/>
-        <v>4.9071507751786703E-2</v>
+        <v>-0.15244060608646604</v>
       </c>
       <c r="AD3" s="5">
         <f t="shared" si="0"/>
@@ -5383,15 +5389,15 @@
       </c>
       <c r="AE3" s="5">
         <f t="shared" si="0"/>
-        <v>-3.590168835295493E-2</v>
+        <v>0.15189914217674877</v>
       </c>
       <c r="AF3" s="5">
         <f t="shared" si="0"/>
-        <v>9.4877074177275589E-6</v>
+        <v>3.0591238866007679E-2</v>
       </c>
       <c r="AG3" s="5">
         <f t="shared" si="0"/>
-        <v>0.16302187076572894</v>
+        <v>0.55986157836480466</v>
       </c>
       <c r="AH3" s="5">
         <f t="shared" si="0"/>
@@ -5399,15 +5405,15 @@
       </c>
       <c r="AI3" s="9">
         <f>AVERAGE(ABS(AA3),ABS(AE3))</f>
-        <v>3.5476247144351575E-2</v>
+        <v>0.1601379482244504</v>
       </c>
       <c r="AJ3" s="9">
         <f t="shared" ref="AJ3:AK17" si="1">AVERAGE(ABS(AB3),ABS(AF3))</f>
-        <v>4.7026684983255494E-3</v>
+        <v>2.1050522671352663E-2</v>
       </c>
       <c r="AK3" s="9">
         <f t="shared" si="1"/>
-        <v>0.10604668925875782</v>
+        <v>0.35615109222563535</v>
       </c>
       <c r="AL3" s="1" t="s">
         <v>23</v>
@@ -5504,43 +5510,43 @@
         <v>-0.190968692302704</v>
       </c>
       <c r="R4" s="14">
-        <v>0.45295586893178053</v>
+        <v>0.25041881136644017</v>
       </c>
       <c r="S4" s="14">
-        <v>8.336256272682778E-2</v>
+        <v>0.1230931391084471</v>
       </c>
       <c r="T4" s="14">
-        <v>1.5780252517185653</v>
+        <v>1.5823909950624377</v>
       </c>
       <c r="U4" s="14">
         <v>1.5707963267948966</v>
       </c>
       <c r="V4" s="14">
-        <v>0.64275082172063169</v>
+        <v>0.43891091109931513</v>
       </c>
       <c r="W4" s="14">
-        <v>2.4290449442103752E-2</v>
+        <v>2.0000001007548257E-2</v>
       </c>
       <c r="X4" s="14">
-        <v>4.6985016730305746</v>
+        <v>4.6939303970820498</v>
       </c>
       <c r="Y4" s="14">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z4" s="15">
-        <v>3.7486559566318778E-6</v>
+        <v>1.9831796074755143E-6</v>
       </c>
       <c r="AA4" s="14">
         <f t="shared" si="0"/>
-        <v>-4.7044131068219475E-2</v>
+        <v>-0.24958118863355983</v>
       </c>
       <c r="AB4" s="14">
         <f t="shared" si="0"/>
-        <v>-3.6637437273172216E-2</v>
+        <v>3.0931391084471072E-3</v>
       </c>
       <c r="AC4" s="14">
         <f t="shared" si="0"/>
-        <v>8.0252517185652739E-3</v>
+        <v>1.2390995062437682E-2</v>
       </c>
       <c r="AD4" s="14">
         <f t="shared" si="0"/>
@@ -5548,15 +5554,15 @@
       </c>
       <c r="AE4" s="14">
         <f t="shared" si="0"/>
-        <v>-5.7249178279368262E-2</v>
+        <v>-0.26108908890068483</v>
       </c>
       <c r="AF4" s="14">
         <f t="shared" si="0"/>
-        <v>-3.570955055789625E-2</v>
+        <v>-3.9999998992451741E-2</v>
       </c>
       <c r="AG4" s="14">
         <f t="shared" si="0"/>
-        <v>-1.3498326969425101E-2</v>
+        <v>-1.8069602917949901E-2</v>
       </c>
       <c r="AH4" s="14">
         <f t="shared" si="0"/>
@@ -5564,27 +5570,27 @@
       </c>
       <c r="AI4" s="16">
         <f t="shared" ref="AI4:AI17" si="2">AVERAGE(ABS(AA4),ABS(AE4))</f>
-        <v>5.2146654673793869E-2</v>
+        <v>0.25533513876712233</v>
       </c>
       <c r="AJ4" s="16">
         <f t="shared" si="1"/>
-        <v>3.6173493915534233E-2</v>
+        <v>2.1546569050449424E-2</v>
       </c>
       <c r="AK4" s="16">
         <f t="shared" si="1"/>
-        <v>1.0761789343995187E-2</v>
+        <v>1.5230298990193791E-2</v>
       </c>
       <c r="AL4" s="8" cm="1">
         <f t="array" ref="AL4">AVERAGE(ABS(AA3:AA17))</f>
-        <v>0.10875581998903511</v>
+        <v>0.11468345431288035</v>
       </c>
       <c r="AM4" s="8" cm="1">
         <f t="array" ref="AM4">AVERAGE(ABS(AB3:AB17))</f>
-        <v>1.2408809674892564E-2</v>
+        <v>6.425773304628536E-3</v>
       </c>
       <c r="AN4" s="8" cm="1">
         <f t="array" ref="AN4">AVERAGE(ABS(AC3:AC17))</f>
-        <v>0.26855322373524426</v>
+        <v>0.38725654397153331</v>
       </c>
       <c r="AO4" s="8" cm="1">
         <f t="array" ref="AO4">AVERAGE(ABS(AD3:AD17))</f>
@@ -5592,15 +5598,15 @@
       </c>
       <c r="AP4" s="8" cm="1">
         <f t="array" ref="AP4">AVERAGE(ABS(AE3:AE17))</f>
-        <v>0.15177723389536327</v>
+        <v>0.12958062342130677</v>
       </c>
       <c r="AQ4" s="8" cm="1">
         <f t="array" ref="AQ4">AVERAGE(ABS(AF3:AF17))</f>
-        <v>1.5460665283895706E-2</v>
+        <v>1.8437226754856727E-2</v>
       </c>
       <c r="AR4" s="8" cm="1">
         <f t="array" ref="AR4">AVERAGE(ABS(AG3:AG17))</f>
-        <v>0.11680568958632016</v>
+        <v>0.16491136013327951</v>
       </c>
       <c r="AS4" s="8" cm="1">
         <f t="array" ref="AS4">AVERAGE(ABS(AH3:AH17))</f>
@@ -5677,43 +5683,43 @@
         <v>0.28356426954269398</v>
       </c>
       <c r="R5" s="5">
-        <v>0.94551212918129546</v>
+        <v>0.94502488529732842</v>
       </c>
       <c r="S5" s="5">
-        <v>0.17370533462932519</v>
+        <v>0.17432651216985234</v>
       </c>
       <c r="T5" s="5">
-        <v>1.60053519576169</v>
+        <v>1.6032158861550252</v>
       </c>
       <c r="U5" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V5" s="5">
-        <v>0.45037434758236827</v>
+        <v>0.44751642356693089</v>
       </c>
       <c r="W5" s="5">
-        <v>8.1459899529797444E-2</v>
+        <v>8.291167043607317E-2</v>
       </c>
       <c r="X5" s="5">
-        <v>4.7635012537812669</v>
+        <v>4.7702810933248534</v>
       </c>
       <c r="Y5" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z5" s="12">
-        <v>1.8978163258711729E-5</v>
+        <v>1.0163531846115792E-5</v>
       </c>
       <c r="AA5" s="5">
         <f t="shared" si="0"/>
-        <v>0.14551212918129541</v>
+        <v>0.14502488529732838</v>
       </c>
       <c r="AB5" s="5">
         <f t="shared" si="0"/>
-        <v>-6.2946653706748013E-3</v>
+        <v>-5.6734878301476499E-3</v>
       </c>
       <c r="AC5" s="5">
         <f t="shared" si="0"/>
-        <v>3.0535195761689948E-2</v>
+        <v>3.3215886155025132E-2</v>
       </c>
       <c r="AD5" s="5">
         <f t="shared" si="0"/>
@@ -5721,15 +5727,15 @@
       </c>
       <c r="AE5" s="5">
         <f t="shared" si="0"/>
-        <v>5.0374347582368251E-2</v>
+        <v>4.7516423566930865E-2</v>
       </c>
       <c r="AF5" s="5">
         <f t="shared" si="0"/>
-        <v>1.4598995297974426E-3</v>
+        <v>2.9116704360731688E-3</v>
       </c>
       <c r="AG5" s="5">
         <f t="shared" si="0"/>
-        <v>5.1501253781267131E-2</v>
+        <v>5.828109332485365E-2</v>
       </c>
       <c r="AH5" s="5">
         <f t="shared" si="0"/>
@@ -5737,26 +5743,26 @@
       </c>
       <c r="AI5" s="9">
         <f t="shared" si="2"/>
-        <v>9.7943238381831832E-2</v>
+        <v>9.6270654432129621E-2</v>
       </c>
       <c r="AJ5" s="9">
         <f t="shared" si="1"/>
-        <v>3.8772824502361219E-3</v>
+        <v>4.2925791331104093E-3</v>
       </c>
       <c r="AK5" s="9">
         <f t="shared" si="1"/>
-        <v>4.101822477147854E-2</v>
-      </c>
-      <c r="AL5" s="30" t="s">
+        <v>4.5748489739939391E-2</v>
+      </c>
+      <c r="AL5" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="AM5" s="30"/>
-      <c r="AN5" s="30"/>
-      <c r="AO5" s="30"/>
-      <c r="AP5" s="30"/>
-      <c r="AQ5" s="30"/>
-      <c r="AR5" s="30"/>
-      <c r="AS5" s="30"/>
+      <c r="AM5" s="31"/>
+      <c r="AN5" s="31"/>
+      <c r="AO5" s="31"/>
+      <c r="AP5" s="31"/>
+      <c r="AQ5" s="31"/>
+      <c r="AR5" s="31"/>
+      <c r="AS5" s="31"/>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
@@ -5828,43 +5834,43 @@
         <v>0.13295280933380099</v>
       </c>
       <c r="R6" s="5">
-        <v>0.30138395208062263</v>
+        <v>0.30132996688458252</v>
       </c>
       <c r="S6" s="5">
-        <v>0.19705670406443784</v>
+        <v>0.19670276251491342</v>
       </c>
       <c r="T6" s="5">
-        <v>1.4640146948999122</v>
+        <v>1.4777144572087972</v>
       </c>
       <c r="U6" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V6" s="5">
-        <v>0.71824829865091189</v>
+        <v>0.71430463741055017</v>
       </c>
       <c r="W6" s="5">
-        <v>5.1420659106028721E-2</v>
+        <v>5.0668780725793297E-2</v>
       </c>
       <c r="X6" s="5">
-        <v>3.3402763911202342</v>
+        <v>3.3428216273501956</v>
       </c>
       <c r="Y6" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z6" s="12">
-        <v>6.9264733304223934E-6</v>
+        <v>3.6905569985762581E-6</v>
       </c>
       <c r="AA6" s="5">
         <f t="shared" si="0"/>
-        <v>1.3839520806226413E-3</v>
+        <v>1.3299668845825341E-3</v>
       </c>
       <c r="AB6" s="5">
         <f t="shared" si="0"/>
-        <v>-2.943295935562168E-3</v>
+        <v>-3.2972374850865904E-3</v>
       </c>
       <c r="AC6" s="5">
         <f t="shared" si="0"/>
-        <v>-0.10598530510008786</v>
+        <v>-9.2285542791202824E-2</v>
       </c>
       <c r="AD6" s="5">
         <f t="shared" si="0"/>
@@ -5872,15 +5878,15 @@
       </c>
       <c r="AE6" s="5">
         <f t="shared" si="0"/>
-        <v>1.8248298650911932E-2</v>
+        <v>1.4304637410550214E-2</v>
       </c>
       <c r="AF6" s="5">
         <f t="shared" si="0"/>
-        <v>1.142065910602872E-2</v>
+        <v>1.0668780725793296E-2</v>
       </c>
       <c r="AG6" s="5">
         <f t="shared" si="0"/>
-        <v>0.19827639112023432</v>
+        <v>0.20082162735019571</v>
       </c>
       <c r="AH6" s="5">
         <f t="shared" si="0"/>
@@ -5888,15 +5894,15 @@
       </c>
       <c r="AI6" s="9">
         <f t="shared" si="2"/>
-        <v>9.8161253657672864E-3</v>
+        <v>7.817302147566374E-3</v>
       </c>
       <c r="AJ6" s="9">
         <f t="shared" si="1"/>
-        <v>7.1819775207954441E-3</v>
+        <v>6.9830091054399433E-3</v>
       </c>
       <c r="AK6" s="9">
         <f t="shared" si="1"/>
-        <v>0.15213084811016109</v>
+        <v>0.14655358507069927</v>
       </c>
       <c r="AL6" s="7" t="s">
         <v>33</v>
@@ -5983,43 +5989,43 @@
         <v>-0.48219949007034302</v>
       </c>
       <c r="R7" s="5">
-        <v>0.52289293380125046</v>
+        <v>0.6007238412725272</v>
       </c>
       <c r="S7" s="5">
-        <v>9.683808059827928E-2</v>
+        <v>9.2515604492737269E-2</v>
       </c>
       <c r="T7" s="5">
-        <v>3.4082518802200492</v>
+        <v>3.0492690320015412</v>
       </c>
       <c r="U7" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V7" s="5">
-        <v>0.53361402151263604</v>
+        <v>0.6273733852419906</v>
       </c>
       <c r="W7" s="5">
-        <v>8.125767348174448E-2</v>
+        <v>8.600955367547386E-2</v>
       </c>
       <c r="X7" s="5">
-        <v>3.8731405691951282</v>
+        <v>4.2118714043553762</v>
       </c>
       <c r="Y7" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z7" s="12">
-        <v>6.1657186592090775E-6</v>
+        <v>3.4221134297188575E-6</v>
       </c>
       <c r="AA7" s="5">
         <f t="shared" si="0"/>
-        <v>0.22289293380125047</v>
+        <v>0.30072384127252721</v>
       </c>
       <c r="AB7" s="5">
         <f t="shared" si="0"/>
-        <v>-3.1619194017207253E-3</v>
+        <v>-7.4843955072627366E-3</v>
       </c>
       <c r="AC7" s="5">
         <f t="shared" si="0"/>
-        <v>0.26625188022004931</v>
+        <v>-9.2730967998458702E-2</v>
       </c>
       <c r="AD7" s="5">
         <f t="shared" si="0"/>
@@ -6027,15 +6033,15 @@
       </c>
       <c r="AE7" s="5">
         <f t="shared" si="0"/>
-        <v>-0.26638597848736401</v>
+        <v>-0.17262661475800944</v>
       </c>
       <c r="AF7" s="5">
         <f t="shared" si="0"/>
-        <v>1.2576734817444785E-3</v>
+        <v>6.0095536754738582E-3</v>
       </c>
       <c r="AG7" s="5">
         <f t="shared" si="0"/>
-        <v>-5.3859430804871877E-2</v>
+        <v>0.28487140435537617</v>
       </c>
       <c r="AH7" s="5">
         <f t="shared" si="0"/>
@@ -6043,27 +6049,27 @@
       </c>
       <c r="AI7" s="9">
         <f t="shared" si="2"/>
-        <v>0.24463945614430724</v>
+        <v>0.23667522801526833</v>
       </c>
       <c r="AJ7" s="9">
         <f t="shared" si="1"/>
-        <v>2.2097964417326019E-3</v>
+        <v>6.7469745913682974E-3</v>
       </c>
       <c r="AK7" s="9">
         <f t="shared" si="1"/>
-        <v>0.16005565551246059</v>
+        <v>0.18880118617691743</v>
       </c>
       <c r="AL7" s="11">
         <f>AVERAGE(AL4,AP4)</f>
-        <v>0.1302665269421992</v>
+        <v>0.12213203886709356</v>
       </c>
       <c r="AM7" s="11">
         <f>AVERAGE(AM4,AQ4)</f>
-        <v>1.3934737479394135E-2</v>
+        <v>1.2431500029742632E-2</v>
       </c>
       <c r="AN7" s="11">
         <f>AVERAGE(AN4,AR4)</f>
-        <v>0.19267945666078221</v>
+        <v>0.27608395205240643</v>
       </c>
       <c r="AO7" s="8"/>
       <c r="AP7" s="8"/>
@@ -6141,43 +6147,43 @@
         <v>-0.22229230403900099</v>
       </c>
       <c r="R8" s="5">
-        <v>0.22585846929220876</v>
+        <v>0.79198522199752341</v>
       </c>
       <c r="S8" s="5">
-        <v>0.14652385779443095</v>
+        <v>9.7214985461209283E-2</v>
       </c>
       <c r="T8" s="5">
-        <v>2.8694937721604359</v>
+        <v>2.9057305409617489</v>
       </c>
       <c r="U8" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V8" s="5">
-        <v>0.91536177013515352</v>
+        <v>0.51704410052088723</v>
       </c>
       <c r="W8" s="5">
-        <v>7.6147256897794321E-2</v>
+        <v>7.3705317327131176E-2</v>
       </c>
       <c r="X8" s="5">
-        <v>3.4535909824894375</v>
+        <v>4.0498926892873603</v>
       </c>
       <c r="Y8" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z8" s="12">
-        <v>3.0325798590758987E-6</v>
+        <v>1.8200446184710511E-6</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="0"/>
-        <v>-0.47414153070779119</v>
+        <v>9.1985221997523459E-2</v>
       </c>
       <c r="AB8" s="5">
         <f t="shared" si="0"/>
-        <v>4.6523857794430939E-2</v>
+        <v>-2.7850145387907227E-3</v>
       </c>
       <c r="AC8" s="5">
         <f t="shared" si="0"/>
-        <v>-0.27250622783956402</v>
+        <v>-0.23626945903825103</v>
       </c>
       <c r="AD8" s="5">
         <f t="shared" si="0"/>
@@ -6185,15 +6191,15 @@
       </c>
       <c r="AE8" s="5">
         <f t="shared" si="0"/>
-        <v>0.5153617701351535</v>
+        <v>0.11704410052088721</v>
       </c>
       <c r="AF8" s="5">
         <f t="shared" si="0"/>
-        <v>3.6147256897794321E-2</v>
+        <v>3.3705317327131175E-2</v>
       </c>
       <c r="AG8" s="5">
         <f t="shared" si="0"/>
-        <v>-0.47340901751056252</v>
+        <v>0.1228926892873603</v>
       </c>
       <c r="AH8" s="5">
         <f t="shared" si="0"/>
@@ -6201,15 +6207,15 @@
       </c>
       <c r="AI8" s="10">
         <f t="shared" si="2"/>
-        <v>0.49475165042147234</v>
+        <v>0.10451466125920533</v>
       </c>
       <c r="AJ8" s="10">
         <f t="shared" si="1"/>
-        <v>4.1335557346112634E-2</v>
+        <v>1.8245165932960949E-2</v>
       </c>
       <c r="AK8" s="10">
         <f t="shared" si="1"/>
-        <v>0.37295762267506327</v>
+        <v>0.17958107416280567</v>
       </c>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.25">
@@ -6282,43 +6288,43 @@
         <v>-0.380674779415131</v>
       </c>
       <c r="R9" s="5">
-        <v>0.58036382003897147</v>
+        <v>0.58717756770531981</v>
       </c>
       <c r="S9" s="5">
-        <v>0.14532857187416842</v>
+        <v>0.14445267408978171</v>
       </c>
       <c r="T9" s="5">
-        <v>3.2124008455685962</v>
+        <v>3.2194164152875895</v>
       </c>
       <c r="U9" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V9" s="5">
-        <v>0.56646971235920485</v>
+        <v>0.5581241517743053</v>
       </c>
       <c r="W9" s="5">
-        <v>8.6797073278955209E-2</v>
+        <v>8.688377484189129E-2</v>
       </c>
       <c r="X9" s="5">
-        <v>3.8118639621024735</v>
+        <v>3.8110322126603302</v>
       </c>
       <c r="Y9" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z9" s="12">
-        <v>2.5724568438911729E-6</v>
+        <v>2.1924955067732803E-6</v>
       </c>
       <c r="AA9" s="5">
         <f t="shared" si="0"/>
-        <v>8.0363820038971467E-2</v>
+        <v>8.7177567705319814E-2</v>
       </c>
       <c r="AB9" s="5">
         <f t="shared" si="0"/>
-        <v>5.3285718741684085E-3</v>
+        <v>4.4526740897816997E-3</v>
       </c>
       <c r="AC9" s="5">
         <f t="shared" si="0"/>
-        <v>7.0400845568596271E-2</v>
+        <v>7.7416415287589579E-2</v>
       </c>
       <c r="AD9" s="5">
         <f t="shared" si="0"/>
@@ -6326,15 +6332,15 @@
       </c>
       <c r="AE9" s="5">
         <f t="shared" si="0"/>
-        <v>-0.13353028764079511</v>
+        <v>-0.14187584822569466</v>
       </c>
       <c r="AF9" s="5">
         <f t="shared" si="0"/>
-        <v>6.7970732789552069E-3</v>
+        <v>6.8837748418912881E-3</v>
       </c>
       <c r="AG9" s="5">
         <f t="shared" si="0"/>
-        <v>-0.11513603789752658</v>
+        <v>-0.11596778733966984</v>
       </c>
       <c r="AH9" s="5">
         <f t="shared" si="0"/>
@@ -6342,15 +6348,15 @@
       </c>
       <c r="AI9" s="9">
         <f t="shared" si="2"/>
-        <v>0.10694705383988329</v>
+        <v>0.11452670796550724</v>
       </c>
       <c r="AJ9" s="9">
         <f t="shared" si="1"/>
-        <v>6.0628225765618077E-3</v>
+        <v>5.6682244658364939E-3</v>
       </c>
       <c r="AK9" s="9">
         <f t="shared" si="1"/>
-        <v>9.2768441733061424E-2</v>
+        <v>9.6692101313629708E-2</v>
       </c>
     </row>
     <row r="10" spans="1:45" x14ac:dyDescent="0.25">
@@ -6423,43 +6429,43 @@
         <v>-0.296476870775223</v>
       </c>
       <c r="R10" s="5">
-        <v>0.71638030975061862</v>
+        <v>0.73069189969582482</v>
       </c>
       <c r="S10" s="5">
-        <v>0.14350431964412669</v>
+        <v>0.14246436187170905</v>
       </c>
       <c r="T10" s="5">
-        <v>3.1358170417740201</v>
+        <v>3.1478032810434784</v>
       </c>
       <c r="U10" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V10" s="5">
-        <v>0.4681031435348918</v>
+        <v>0.45105356306419725</v>
       </c>
       <c r="W10" s="5">
-        <v>7.6234715125892763E-2</v>
+        <v>7.5369332742168393E-2</v>
       </c>
       <c r="X10" s="5">
-        <v>3.8492952607801145</v>
+        <v>3.8528750760077211</v>
       </c>
       <c r="Y10" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z10" s="12">
-        <v>5.0031203443924436E-6</v>
+        <v>3.2487021033480912E-6</v>
       </c>
       <c r="AA10" s="5">
         <f t="shared" si="0"/>
-        <v>1.638030975061866E-2</v>
+        <v>3.0691899695824865E-2</v>
       </c>
       <c r="AB10" s="5">
         <f t="shared" si="0"/>
-        <v>3.5043196441266744E-3</v>
+        <v>2.4643618717090365E-3</v>
       </c>
       <c r="AC10" s="5">
         <f t="shared" si="0"/>
-        <v>-6.1829582259798066E-3</v>
+        <v>5.8032810434784921E-3</v>
       </c>
       <c r="AD10" s="5">
         <f t="shared" si="0"/>
@@ -6467,15 +6473,15 @@
       </c>
       <c r="AE10" s="5">
         <f t="shared" si="0"/>
-        <v>-3.1896856465108203E-2</v>
+        <v>-4.8946436935802751E-2</v>
       </c>
       <c r="AF10" s="5">
         <f t="shared" si="0"/>
-        <v>1.6234715125892765E-2</v>
+        <v>1.5369332742168396E-2</v>
       </c>
       <c r="AG10" s="5">
         <f t="shared" si="0"/>
-        <v>-7.7704739219885521E-2</v>
+        <v>-7.412492399227899E-2</v>
       </c>
       <c r="AH10" s="5">
         <f t="shared" si="0"/>
@@ -6483,15 +6489,15 @@
       </c>
       <c r="AI10" s="9">
         <f t="shared" si="2"/>
-        <v>2.4138583107863432E-2</v>
+        <v>3.9819168315813808E-2</v>
       </c>
       <c r="AJ10" s="9">
         <f t="shared" si="1"/>
-        <v>9.8695173850097198E-3</v>
+        <v>8.9168473069387161E-3</v>
       </c>
       <c r="AK10" s="9">
         <f t="shared" si="1"/>
-        <v>4.1943848722932664E-2</v>
+        <v>3.9964102517878741E-2</v>
       </c>
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.25">
@@ -6564,43 +6570,43 @@
         <v>-0.23403739929199199</v>
       </c>
       <c r="R11" s="5">
-        <v>0.39115139394893778</v>
+        <v>0.38144916064868661</v>
       </c>
       <c r="S11" s="5">
-        <v>0.17848613232598826</v>
+        <v>0.1815825776163196</v>
       </c>
       <c r="T11" s="5">
-        <v>3.1553352325056365</v>
+        <v>3.1528301989041752</v>
       </c>
       <c r="U11" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V11" s="5">
-        <v>0.3376916900981245</v>
+        <v>0.34637285207868712</v>
       </c>
       <c r="W11" s="5">
-        <v>2.6753075845865247E-2</v>
+        <v>2.7472351559962548E-2</v>
       </c>
       <c r="X11" s="5">
-        <v>3.8761623796876643</v>
+        <v>3.8575241813413221</v>
       </c>
       <c r="Y11" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z11" s="12">
-        <v>3.0215967247152278E-6</v>
+        <v>2.1133239082224754E-6</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="0"/>
-        <v>-8.8486060510622466E-3</v>
+        <v>-1.8550839351313408E-2</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="0"/>
-        <v>-1.5138676740117374E-3</v>
+        <v>1.5825776163196081E-3</v>
       </c>
       <c r="AC11" s="5">
         <f t="shared" si="0"/>
-        <v>1.3335232505636618E-2</v>
+        <v>1.0830198904175248E-2</v>
       </c>
       <c r="AD11" s="5">
         <f t="shared" si="0"/>
@@ -6608,15 +6614,15 @@
       </c>
       <c r="AE11" s="5">
         <f t="shared" si="0"/>
-        <v>-6.2308309901875525E-2</v>
+        <v>-5.3627147921312901E-2</v>
       </c>
       <c r="AF11" s="5">
         <f t="shared" si="0"/>
-        <v>6.7530758458652466E-3</v>
+        <v>7.4723515599625472E-3</v>
       </c>
       <c r="AG11" s="5">
         <f t="shared" si="0"/>
-        <v>-5.0837620312335741E-2</v>
+        <v>-6.9475818658677913E-2</v>
       </c>
       <c r="AH11" s="5">
         <f t="shared" si="0"/>
@@ -6624,15 +6630,15 @@
       </c>
       <c r="AI11" s="9">
         <f t="shared" si="2"/>
-        <v>3.5578457976468886E-2</v>
+        <v>3.6088993636313155E-2</v>
       </c>
       <c r="AJ11" s="9">
         <f t="shared" si="1"/>
-        <v>4.133471759938492E-3</v>
+        <v>4.5274645881410776E-3</v>
       </c>
       <c r="AK11" s="9">
         <f t="shared" si="1"/>
-        <v>3.2086426408986179E-2</v>
+        <v>4.015300878142658E-2</v>
       </c>
     </row>
     <row r="12" spans="1:45" x14ac:dyDescent="0.25">
@@ -6705,43 +6711,43 @@
         <v>-0.46333062648773199</v>
       </c>
       <c r="R12" s="5">
-        <v>0.95500777035355255</v>
+        <v>0.95477462037983485</v>
       </c>
       <c r="S12" s="5">
-        <v>0.16187131340355476</v>
+        <v>0.16173925574813475</v>
       </c>
       <c r="T12" s="5">
-        <v>3.2004098840767701</v>
+        <v>3.2005032099253139</v>
       </c>
       <c r="U12" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V12" s="5">
-        <v>0.56929918428276849</v>
+        <v>0.56866290861468605</v>
       </c>
       <c r="W12" s="5">
-        <v>3.8310976199279478E-2</v>
+        <v>3.8612452870769476E-2</v>
       </c>
       <c r="X12" s="5">
-        <v>3.9543421549541562</v>
+        <v>3.9539774089694384</v>
       </c>
       <c r="Y12" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z12" s="12">
-        <v>1.3946083844033257E-5</v>
+        <v>8.0938724382109526E-6</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="0"/>
-        <v>0.2550077703535526</v>
+        <v>0.25477462037983489</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="0"/>
-        <v>-1.8128686596445232E-2</v>
+        <v>-1.8260744251865246E-2</v>
       </c>
       <c r="AC12" s="5">
         <f t="shared" si="0"/>
-        <v>5.8409884076770169E-2</v>
+        <v>5.8503209925313993E-2</v>
       </c>
       <c r="AD12" s="5">
         <f t="shared" si="0"/>
@@ -6749,15 +6755,15 @@
       </c>
       <c r="AE12" s="5">
         <f t="shared" si="0"/>
-        <v>-0.23070081571723156</v>
+        <v>-0.231337091385314</v>
       </c>
       <c r="AF12" s="5">
         <f t="shared" si="0"/>
-        <v>-1.6890238007205224E-3</v>
+        <v>-1.387547129230525E-3</v>
       </c>
       <c r="AG12" s="5">
         <f t="shared" si="0"/>
-        <v>2.734215495415615E-2</v>
+        <v>2.6977408969438343E-2</v>
       </c>
       <c r="AH12" s="5">
         <f t="shared" si="0"/>
@@ -6765,15 +6771,15 @@
       </c>
       <c r="AI12" s="9">
         <f t="shared" si="2"/>
-        <v>0.24285429303539208</v>
+        <v>0.24305585588257445</v>
       </c>
       <c r="AJ12" s="9">
         <f t="shared" si="1"/>
-        <v>9.908855198582877E-3</v>
+        <v>9.8241456905478856E-3</v>
       </c>
       <c r="AK12" s="9">
         <f t="shared" si="1"/>
-        <v>4.287601951546316E-2</v>
+        <v>4.2740309447376168E-2</v>
       </c>
     </row>
     <row r="13" spans="1:45" x14ac:dyDescent="0.25">
@@ -6846,43 +6852,43 @@
         <v>-0.59106355905532804</v>
       </c>
       <c r="R13" s="5">
-        <v>0.22895453303777191</v>
+        <v>0.18389499419071753</v>
       </c>
       <c r="S13" s="5">
-        <v>9.2425680402638849E-2</v>
+        <v>0.10100790522659002</v>
       </c>
       <c r="T13" s="5">
-        <v>1.9435175511633407</v>
+        <v>0.10508399434679921</v>
       </c>
       <c r="U13" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V13" s="5">
-        <v>0.80200266584895874</v>
+        <v>0.64992094155221658</v>
       </c>
       <c r="W13" s="5">
-        <v>9.0845807363278352E-2</v>
+        <v>9.1077969828068789E-2</v>
       </c>
       <c r="X13" s="5">
-        <v>4.7613997274183504</v>
+        <v>4.3422649428357536</v>
       </c>
       <c r="Y13" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z13" s="12">
-        <v>4.5058826258141946E-6</v>
+        <v>2.3932453890050979E-6</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="0"/>
-        <v>-7.1045466962228077E-2</v>
+        <v>-0.11610500580928246</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="0"/>
-        <v>-2.7574319597361147E-2</v>
+        <v>-1.8992094773409976E-2</v>
       </c>
       <c r="AC13" s="5">
         <f t="shared" si="0"/>
-        <v>-2.7684824488366591</v>
+        <v>-4.6069160056532006</v>
       </c>
       <c r="AD13" s="5">
         <f t="shared" si="0"/>
@@ -6890,15 +6896,15 @@
       </c>
       <c r="AE13" s="5">
         <f t="shared" si="0"/>
-        <v>0.5020026658489587</v>
+        <v>0.34992094155221659</v>
       </c>
       <c r="AF13" s="5">
         <f t="shared" si="0"/>
-        <v>5.0845807363278352E-2</v>
+        <v>5.1077969828068788E-2</v>
       </c>
       <c r="AG13" s="5">
         <f t="shared" si="0"/>
-        <v>4.9399727418350636E-2</v>
+        <v>-0.36973505716424615</v>
       </c>
       <c r="AH13" s="5">
         <f t="shared" si="0"/>
@@ -6906,15 +6912,15 @@
       </c>
       <c r="AI13" s="9">
         <f t="shared" si="2"/>
-        <v>0.28652406640559336</v>
+        <v>0.23301297368074952</v>
       </c>
       <c r="AJ13" s="9">
         <f t="shared" si="1"/>
-        <v>3.9210063480319746E-2</v>
+        <v>3.5035032300739385E-2</v>
       </c>
       <c r="AK13" s="9">
         <f t="shared" si="1"/>
-        <v>1.4089410881275048</v>
+        <v>2.4883255314087234</v>
       </c>
     </row>
     <row r="14" spans="1:45" x14ac:dyDescent="0.25">
@@ -6987,43 +6993,43 @@
         <v>-0.86990654468536399</v>
       </c>
       <c r="R14" s="5">
-        <v>0.90114115674254114</v>
+        <v>0.84892738150496216</v>
       </c>
       <c r="S14" s="5">
-        <v>0.12212369847926889</v>
+        <v>0.12754331454010301</v>
       </c>
       <c r="T14" s="5">
-        <v>4.7879032099079879</v>
+        <v>4.7942787408862424</v>
       </c>
       <c r="U14" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V14" s="5">
-        <v>0.77076018971583138</v>
+        <v>0.77533575200178861</v>
       </c>
       <c r="W14" s="5">
-        <v>3.3442190427954335E-2</v>
+        <v>3.4057077790632481E-2</v>
       </c>
       <c r="X14" s="5">
-        <v>3.1657457889830156</v>
+        <v>3.2362002577942977</v>
       </c>
       <c r="Y14" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z14" s="12">
-        <v>5.2721899592441147E-6</v>
+        <v>2.8667231543968942E-6</v>
       </c>
       <c r="AA14" s="5">
         <f t="shared" si="0"/>
-        <v>0.10114115674254109</v>
+        <v>4.892738150496212E-2</v>
       </c>
       <c r="AB14" s="5">
         <f t="shared" si="0"/>
-        <v>2.1236984792688957E-3</v>
+        <v>7.5433145401030133E-3</v>
       </c>
       <c r="AC14" s="5">
         <f t="shared" si="0"/>
-        <v>7.5903209907988156E-2</v>
+        <v>8.2278740886242652E-2</v>
       </c>
       <c r="AD14" s="5">
         <f t="shared" si="0"/>
@@ -7031,15 +7037,15 @@
       </c>
       <c r="AE14" s="5">
         <f t="shared" si="0"/>
-        <v>7.0760189715831423E-2</v>
+        <v>7.5335752001788658E-2</v>
       </c>
       <c r="AF14" s="5">
         <f t="shared" si="0"/>
-        <v>1.3442190427954335E-2</v>
+        <v>1.4057077790632481E-2</v>
       </c>
       <c r="AG14" s="5">
         <f t="shared" si="0"/>
-        <v>2.3745788983015714E-2</v>
+        <v>9.4200257794297748E-2</v>
       </c>
       <c r="AH14" s="5">
         <f t="shared" si="0"/>
@@ -7047,15 +7053,15 @@
       </c>
       <c r="AI14" s="9">
         <f t="shared" si="2"/>
-        <v>8.5950673229186259E-2</v>
+        <v>6.2131566753375389E-2</v>
       </c>
       <c r="AJ14" s="9">
         <f t="shared" si="1"/>
-        <v>7.7829444536116153E-3</v>
+        <v>1.0800196165367747E-2</v>
       </c>
       <c r="AK14" s="9">
         <f t="shared" si="1"/>
-        <v>4.9824499445501935E-2</v>
+        <v>8.82394993402702E-2</v>
       </c>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.25">
@@ -7128,43 +7134,43 @@
         <v>-0.37272521853446999</v>
       </c>
       <c r="R15" s="5">
-        <v>0.39029559980793083</v>
+        <v>0.37162833410010049</v>
       </c>
       <c r="S15" s="5">
-        <v>0.17939657912288887</v>
+        <v>0.1855889089114266</v>
       </c>
       <c r="T15" s="5">
-        <v>4.77524333088909</v>
+        <v>4.7806231137486623</v>
       </c>
       <c r="U15" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V15" s="5">
-        <v>0.52073102586095477</v>
+        <v>0.52257591038996165</v>
       </c>
       <c r="W15" s="5">
-        <v>6.6167145645490449E-2</v>
+        <v>6.6545551554697144E-2</v>
       </c>
       <c r="X15" s="5">
-        <v>3.1652411388562318</v>
+        <v>3.20079696238041</v>
       </c>
       <c r="Y15" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z15" s="12">
-        <v>4.1341226486663472E-6</v>
+        <v>2.5698174118158339E-6</v>
       </c>
       <c r="AA15" s="5">
         <f t="shared" si="0"/>
-        <v>-9.7044001920691958E-3</v>
+        <v>-2.8371665899899534E-2</v>
       </c>
       <c r="AB15" s="5">
         <f t="shared" si="0"/>
-        <v>-6.0342087711112713E-4</v>
+        <v>5.5889089114266044E-3</v>
       </c>
       <c r="AC15" s="5">
         <f t="shared" si="0"/>
-        <v>6.3243330889090288E-2</v>
+        <v>6.862311374866259E-2</v>
       </c>
       <c r="AD15" s="5">
         <f t="shared" si="0"/>
@@ -7172,15 +7178,15 @@
       </c>
       <c r="AE15" s="5">
         <f t="shared" si="0"/>
-        <v>2.0731025860954766E-2</v>
+        <v>2.2575910389961651E-2</v>
       </c>
       <c r="AF15" s="5">
         <f t="shared" si="0"/>
-        <v>6.1671456454904516E-3</v>
+        <v>6.545551554697146E-3</v>
       </c>
       <c r="AG15" s="5">
         <f t="shared" si="0"/>
-        <v>2.3241138856231913E-2</v>
+        <v>5.87969623804101E-2</v>
       </c>
       <c r="AH15" s="5">
         <f t="shared" si="0"/>
@@ -7188,15 +7194,15 @@
       </c>
       <c r="AI15" s="9">
         <f t="shared" si="2"/>
-        <v>1.5217713026511981E-2</v>
+        <v>2.5473788144930593E-2</v>
       </c>
       <c r="AJ15" s="9">
         <f t="shared" si="1"/>
-        <v>3.3852832613007894E-3</v>
+        <v>6.0672302330618752E-3</v>
       </c>
       <c r="AK15" s="9">
         <f t="shared" si="1"/>
-        <v>4.3242234872661101E-2</v>
+        <v>6.3710038064536345E-2</v>
       </c>
     </row>
     <row r="16" spans="1:45" x14ac:dyDescent="0.25">
@@ -7269,43 +7275,43 @@
         <v>-1.05074739456177</v>
       </c>
       <c r="R16" s="5">
-        <v>0.5319492699732804</v>
+        <v>0.47651184347498193</v>
       </c>
       <c r="S16" s="5">
-        <v>0.17760176561114949</v>
+        <v>0.19634115743164984</v>
       </c>
       <c r="T16" s="5">
-        <v>4.6376371378789347</v>
+        <v>4.6408460246990018</v>
       </c>
       <c r="U16" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V16" s="5">
-        <v>0.55991927009066922</v>
+        <v>0.62656885273157326</v>
       </c>
       <c r="W16" s="5">
         <v>2.0000000000022205E-2</v>
       </c>
       <c r="X16" s="5">
-        <v>4.7214665516405248</v>
+        <v>4.7085885697331307</v>
       </c>
       <c r="Y16" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z16" s="12">
-        <v>1.8974768311189834E-5</v>
+        <v>1.1987718553480196E-5</v>
       </c>
       <c r="AA16" s="5">
         <f t="shared" si="0"/>
-        <v>3.1949269973280403E-2</v>
+        <v>-2.3488156525018067E-2</v>
       </c>
       <c r="AB16" s="5">
         <f t="shared" si="0"/>
-        <v>-2.2398234388850524E-2</v>
+        <v>-3.658842568350168E-3</v>
       </c>
       <c r="AC16" s="5">
         <f t="shared" si="0"/>
-        <v>-7.4362862121065021E-2</v>
+        <v>-7.1153975300997985E-2</v>
       </c>
       <c r="AD16" s="5">
         <f t="shared" si="0"/>
@@ -7313,7 +7319,7 @@
       </c>
       <c r="AE16" s="5">
         <f t="shared" si="0"/>
-        <v>-0.14008072990933074</v>
+        <v>-7.34311472684267E-2</v>
       </c>
       <c r="AF16" s="5">
         <f t="shared" si="0"/>
@@ -7321,7 +7327,7 @@
       </c>
       <c r="AG16" s="5">
         <f t="shared" si="0"/>
-        <v>9.4665516405250116E-3</v>
+        <v>-3.4114302668690755E-3</v>
       </c>
       <c r="AH16" s="5">
         <f t="shared" si="0"/>
@@ -7329,15 +7335,15 @@
       </c>
       <c r="AI16" s="9">
         <f t="shared" si="2"/>
-        <v>8.601499994130557E-2</v>
+        <v>4.8459651896722383E-2</v>
       </c>
       <c r="AJ16" s="9">
         <f t="shared" si="1"/>
-        <v>1.1199117194436364E-2</v>
+        <v>1.8294212841861862E-3</v>
       </c>
       <c r="AK16" s="9">
         <f t="shared" si="1"/>
-        <v>4.1914706880795016E-2</v>
+        <v>3.728270278393353E-2</v>
       </c>
     </row>
     <row r="17" spans="1:37" x14ac:dyDescent="0.25">
@@ -7410,43 +7416,43 @@
         <v>-0.37296327948570301</v>
       </c>
       <c r="R17" s="5">
-        <v>0.83087101699627564</v>
+        <v>0.85514281946407666</v>
       </c>
       <c r="S17" s="5">
-        <v>0.19999999907274948</v>
+        <v>0.19999999999996979</v>
       </c>
       <c r="T17" s="5">
-        <v>4.8776022155051351</v>
+        <v>4.9199897616914967</v>
       </c>
       <c r="U17" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="V17" s="5">
-        <v>0.44112636588224152</v>
+        <v>0.48217906830527207</v>
       </c>
       <c r="W17" s="5">
-        <v>0.1239764204895776</v>
+        <v>0.12987823585324665</v>
       </c>
       <c r="X17" s="5">
-        <v>2.7203547064393145</v>
+        <v>2.725817240167236</v>
       </c>
       <c r="Y17" s="5">
         <v>1.5707963267948966</v>
       </c>
       <c r="Z17" s="12">
-        <v>2.5288064699482858E-5</v>
+        <v>1.3071785454381153E-5</v>
       </c>
       <c r="AA17" s="5">
         <f t="shared" si="0"/>
-        <v>0.13087101699627568</v>
+        <v>0.15514281946407671</v>
       </c>
       <c r="AB17" s="5">
         <f t="shared" si="0"/>
-        <v>-9.2725052636133398E-10</v>
+        <v>-3.0225821845419887E-14</v>
       </c>
       <c r="AC17" s="5">
         <f t="shared" si="0"/>
-        <v>0.16560221550513532</v>
+        <v>0.20798976169149697</v>
       </c>
       <c r="AD17" s="5">
         <f t="shared" si="0"/>
@@ -7454,15 +7460,15 @@
       </c>
       <c r="AE17" s="5">
         <f t="shared" si="0"/>
-        <v>0.14112636588224153</v>
+        <v>0.18217906830527208</v>
       </c>
       <c r="AF17" s="5">
         <f t="shared" si="0"/>
-        <v>4.3976420489577603E-2</v>
+        <v>4.9878235853246647E-2</v>
       </c>
       <c r="AG17" s="5">
         <f t="shared" si="0"/>
-        <v>-0.42164529356068536</v>
+        <v>-0.41618275983276387</v>
       </c>
       <c r="AH17" s="5">
         <f t="shared" si="0"/>
@@ -7470,24 +7476,24 @@
       </c>
       <c r="AI17" s="9">
         <f t="shared" si="2"/>
-        <v>0.13599869143925861</v>
+        <v>0.1686609438846744</v>
       </c>
       <c r="AJ17" s="9">
         <f t="shared" si="1"/>
-        <v>2.1988210708414065E-2</v>
+        <v>2.4939117926638436E-2</v>
       </c>
       <c r="AK17" s="9">
         <f t="shared" si="1"/>
-        <v>0.29362375453291034</v>
+        <v>0.31208626076213042</v>
       </c>
     </row>
     <row r="18" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="38"/>
       <c r="H19" s="1" t="s">
         <v>43</v>
       </c>
@@ -7500,14 +7506,14 @@
       <c r="K19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L19" s="23" t="s">
+      <c r="L19" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="M19" s="24"/>
-      <c r="N19" s="24"/>
-      <c r="O19" s="24"/>
-      <c r="P19" s="24"/>
-      <c r="Q19" s="24"/>
+      <c r="M19" s="25"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
+      <c r="Q19" s="25"/>
     </row>
     <row r="20" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A20">
@@ -9765,10 +9771,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8114305-D99A-4A21-9698-292BE3739741}">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AR10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="S1" s="39" t="s">
         <v>46</v>
       </c>
@@ -9779,8 +9785,28 @@
       <c r="X1" s="39"/>
       <c r="Y1" s="39"/>
       <c r="Z1" s="39"/>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB1" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC1" s="39"/>
+      <c r="AD1" s="39"/>
+      <c r="AE1" s="39"/>
+      <c r="AF1" s="39"/>
+      <c r="AG1" s="39"/>
+      <c r="AH1" s="39"/>
+      <c r="AI1" s="39"/>
+      <c r="AK1" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL1" s="39"/>
+      <c r="AM1" s="39"/>
+      <c r="AN1" s="39"/>
+      <c r="AO1" s="39"/>
+      <c r="AP1" s="39"/>
+      <c r="AQ1" s="39"/>
+      <c r="AR1" s="39"/>
+    </row>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.5</v>
       </c>
@@ -9830,32 +9856,80 @@
         <v>1.5708</v>
       </c>
       <c r="S2">
-        <v>0.46560000000000001</v>
+        <v>0.67879999999999996</v>
       </c>
       <c r="T2">
-        <v>0.12920000000000001</v>
+        <v>0.10730000000000001</v>
       </c>
       <c r="U2">
-        <v>1.6194999999999999</v>
+        <v>1.4238999999999999</v>
       </c>
       <c r="V2">
         <v>1.5708</v>
       </c>
       <c r="W2">
-        <v>0.26390000000000002</v>
+        <v>0.45629999999999998</v>
       </c>
       <c r="X2">
-        <v>0.02</v>
+        <v>4.9799999999999997E-2</v>
       </c>
       <c r="Y2">
-        <v>3.3085</v>
+        <v>3.726</v>
       </c>
       <c r="Z2">
         <v>1.5708</v>
       </c>
-      <c r="AA2" s="40"/>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB2">
+        <v>0.4834</v>
+      </c>
+      <c r="AC2">
+        <v>0.12939999999999999</v>
+      </c>
+      <c r="AD2">
+        <v>1.5504</v>
+      </c>
+      <c r="AE2">
+        <v>1.5708</v>
+      </c>
+      <c r="AF2">
+        <v>0.29749999999999999</v>
+      </c>
+      <c r="AG2">
+        <v>3.39E-2</v>
+      </c>
+      <c r="AH2">
+        <v>3.3673000000000002</v>
+      </c>
+      <c r="AI2">
+        <v>1.5708</v>
+      </c>
+      <c r="AJ2" s="21"/>
+      <c r="AK2">
+        <v>0.4738</v>
+      </c>
+      <c r="AL2">
+        <v>0.13950000000000001</v>
+      </c>
+      <c r="AM2">
+        <v>1.8541000000000001</v>
+      </c>
+      <c r="AN2">
+        <v>1.5708</v>
+      </c>
+      <c r="AO2">
+        <v>0.1</v>
+      </c>
+      <c r="AP2">
+        <v>0.1008</v>
+      </c>
+      <c r="AQ2">
+        <v>5.0019</v>
+      </c>
+      <c r="AR2">
+        <v>1.5708</v>
+      </c>
+    </row>
+    <row r="4" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0.8</v>
       </c>
@@ -9905,32 +9979,81 @@
         <v>1.5708</v>
       </c>
       <c r="S4">
-        <v>0.9456</v>
+        <v>0.91920000000000002</v>
       </c>
       <c r="T4">
-        <v>0.17369999999999999</v>
+        <v>0.1759</v>
       </c>
       <c r="U4">
-        <v>1.6016999999999999</v>
+        <v>1.6021000000000001</v>
       </c>
       <c r="V4">
         <v>1.5708</v>
       </c>
       <c r="W4">
-        <v>0.4506</v>
+        <v>0.4214</v>
       </c>
       <c r="X4">
-        <v>8.14E-2</v>
+        <v>8.1100000000000005E-2</v>
       </c>
       <c r="Y4">
-        <v>4.7667000000000002</v>
+        <v>4.7686000000000002</v>
       </c>
       <c r="Z4">
         <v>1.5708</v>
       </c>
-      <c r="AA4" s="40"/>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AA4" s="21"/>
+      <c r="AB4">
+        <v>0.85260000000000002</v>
+      </c>
+      <c r="AC4">
+        <v>0.1852</v>
+      </c>
+      <c r="AD4">
+        <v>1.6801999999999999</v>
+      </c>
+      <c r="AE4">
+        <v>1.5708</v>
+      </c>
+      <c r="AF4">
+        <v>0.34370000000000001</v>
+      </c>
+      <c r="AG4">
+        <v>8.9300000000000004E-2</v>
+      </c>
+      <c r="AH4">
+        <v>4.9741</v>
+      </c>
+      <c r="AI4">
+        <v>1.5708</v>
+      </c>
+      <c r="AJ4" s="21"/>
+      <c r="AK4">
+        <v>0.57469999999999999</v>
+      </c>
+      <c r="AL4">
+        <v>0.19550000000000001</v>
+      </c>
+      <c r="AM4">
+        <v>1.6729000000000001</v>
+      </c>
+      <c r="AN4">
+        <v>1.5708</v>
+      </c>
+      <c r="AO4">
+        <v>0.1</v>
+      </c>
+      <c r="AP4">
+        <v>0.15709999999999999</v>
+      </c>
+      <c r="AQ4">
+        <v>4.7888999999999999</v>
+      </c>
+      <c r="AR4">
+        <v>1.5708</v>
+      </c>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.3</v>
       </c>
@@ -9980,32 +10103,81 @@
         <v>1.5708</v>
       </c>
       <c r="S6">
-        <v>0.30470000000000003</v>
+        <v>0.29930000000000001</v>
       </c>
       <c r="T6">
-        <v>0.19450000000000001</v>
+        <v>0.19739999999999999</v>
       </c>
       <c r="U6">
-        <v>1.4612000000000001</v>
+        <v>1.4778</v>
       </c>
       <c r="V6">
         <v>1.5708</v>
       </c>
       <c r="W6">
-        <v>0.72009999999999996</v>
+        <v>0.71360000000000001</v>
       </c>
       <c r="X6">
-        <v>5.16E-2</v>
+        <v>5.0700000000000002E-2</v>
       </c>
       <c r="Y6">
-        <v>3.3448000000000002</v>
+        <v>3.34</v>
       </c>
       <c r="Z6">
         <v>1.5708</v>
       </c>
-      <c r="AA6" s="40"/>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AA6" s="21"/>
+      <c r="AB6">
+        <v>0.33029999999999998</v>
+      </c>
+      <c r="AC6">
+        <v>0.19980000000000001</v>
+      </c>
+      <c r="AD6">
+        <v>1.65</v>
+      </c>
+      <c r="AE6">
+        <v>1.5708</v>
+      </c>
+      <c r="AF6">
+        <v>0.66520000000000001</v>
+      </c>
+      <c r="AG6">
+        <v>4.2599999999999999E-2</v>
+      </c>
+      <c r="AH6">
+        <v>3.4403999999999999</v>
+      </c>
+      <c r="AI6">
+        <v>1.5708</v>
+      </c>
+      <c r="AJ6" s="21"/>
+      <c r="AK6">
+        <v>0.63739999999999997</v>
+      </c>
+      <c r="AL6">
+        <v>0.2</v>
+      </c>
+      <c r="AM6">
+        <v>0.9093</v>
+      </c>
+      <c r="AN6">
+        <v>1.5708</v>
+      </c>
+      <c r="AO6">
+        <v>0.93479999999999996</v>
+      </c>
+      <c r="AP6">
+        <v>0.15409999999999999</v>
+      </c>
+      <c r="AQ6">
+        <v>3.4982000000000002</v>
+      </c>
+      <c r="AR6">
+        <v>1.5708</v>
+      </c>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.3</v>
       </c>
@@ -10055,32 +10227,79 @@
         <v>1.5708</v>
       </c>
       <c r="S8">
-        <v>0.62519999999999998</v>
+        <v>0.62629999999999997</v>
       </c>
       <c r="T8">
-        <v>9.2200000000000004E-2</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="U8">
-        <v>3.0066000000000002</v>
+        <v>3.0059</v>
       </c>
       <c r="V8">
         <v>1.5708</v>
       </c>
       <c r="W8">
-        <v>0.64370000000000005</v>
+        <v>0.64319999999999999</v>
       </c>
       <c r="X8">
-        <v>8.6099999999999996E-2</v>
+        <v>8.6400000000000005E-2</v>
       </c>
       <c r="Y8">
-        <v>4.2611999999999997</v>
+        <v>4.2625999999999999</v>
       </c>
       <c r="Z8">
         <v>1.5708</v>
       </c>
-      <c r="AA8" s="41"/>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB8">
+        <v>0.64480000000000004</v>
+      </c>
+      <c r="AC8">
+        <v>9.5899999999999999E-2</v>
+      </c>
+      <c r="AD8">
+        <v>4.2896000000000001</v>
+      </c>
+      <c r="AE8">
+        <v>1.5708</v>
+      </c>
+      <c r="AF8">
+        <v>0.63400000000000001</v>
+      </c>
+      <c r="AG8">
+        <v>9.3200000000000005E-2</v>
+      </c>
+      <c r="AH8">
+        <v>2.9603000000000002</v>
+      </c>
+      <c r="AI8">
+        <v>1.5708</v>
+      </c>
+      <c r="AK8">
+        <v>0.17169999999999999</v>
+      </c>
+      <c r="AL8">
+        <v>0.14169999999999999</v>
+      </c>
+      <c r="AM8">
+        <v>3.9645000000000001</v>
+      </c>
+      <c r="AN8">
+        <v>1.5708</v>
+      </c>
+      <c r="AO8">
+        <v>0.81810000000000005</v>
+      </c>
+      <c r="AP8">
+        <v>9.4399999999999998E-2</v>
+      </c>
+      <c r="AQ8">
+        <v>3.5503999999999998</v>
+      </c>
+      <c r="AR8">
+        <v>1.5708</v>
+      </c>
+    </row>
+    <row r="10" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0.7</v>
       </c>
@@ -10130,34 +10349,84 @@
         <v>1.5708</v>
       </c>
       <c r="S10">
-        <v>0.86850000000000005</v>
+        <v>0.82950000000000002</v>
       </c>
       <c r="T10">
-        <v>0.1038</v>
+        <v>9.6199999999999994E-2</v>
       </c>
       <c r="U10">
-        <v>3.2111000000000001</v>
+        <v>2.8826999999999998</v>
       </c>
       <c r="V10">
         <v>1.5708</v>
       </c>
       <c r="W10">
-        <v>0.27629999999999999</v>
+        <v>0.52059999999999995</v>
       </c>
       <c r="X10">
-        <v>3.7100000000000001E-2</v>
+        <v>7.4499999999999997E-2</v>
       </c>
       <c r="Y10">
-        <v>3.7679999999999998</v>
+        <v>4.1315</v>
       </c>
       <c r="Z10">
         <v>1.5708</v>
       </c>
-      <c r="AA10" s="40"/>
+      <c r="AB10">
+        <v>0.69630000000000003</v>
+      </c>
+      <c r="AC10">
+        <v>0.1169</v>
+      </c>
+      <c r="AD10">
+        <v>3.1819000000000002</v>
+      </c>
+      <c r="AE10">
+        <v>1.5708</v>
+      </c>
+      <c r="AF10">
+        <v>0.44019999999999998</v>
+      </c>
+      <c r="AG10">
+        <v>4.3499999999999997E-2</v>
+      </c>
+      <c r="AH10">
+        <v>3.6049000000000002</v>
+      </c>
+      <c r="AI10">
+        <v>1.5708</v>
+      </c>
+      <c r="AJ10" s="21"/>
+      <c r="AK10">
+        <v>0.64480000000000004</v>
+      </c>
+      <c r="AL10">
+        <v>0.12039999999999999</v>
+      </c>
+      <c r="AM10">
+        <v>3.1659999999999999</v>
+      </c>
+      <c r="AN10">
+        <v>1.5708</v>
+      </c>
+      <c r="AO10">
+        <v>0.49180000000000001</v>
+      </c>
+      <c r="AP10">
+        <v>4.6800000000000001E-2</v>
+      </c>
+      <c r="AQ10">
+        <v>3.5819999999999999</v>
+      </c>
+      <c r="AR10">
+        <v>1.5708</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="S1:Z1"/>
+    <mergeCell ref="AB1:AI1"/>
+    <mergeCell ref="AK1:AR1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10173,22 +10442,22 @@
         <v>39</v>
       </c>
       <c r="B2">
-        <v>-1.4753518626093899E-3</v>
+        <v>-1.37211009860039E-3</v>
       </c>
       <c r="C2">
-        <v>3.1907491385936702E-2</v>
+        <v>8.7113633751869202E-2</v>
       </c>
       <c r="D2">
-        <v>-0.19490382075309801</v>
+        <v>-0.16279363632202101</v>
       </c>
       <c r="E2">
-        <v>-0.17070601880550401</v>
+        <v>-9.0744964778423295E-2</v>
       </c>
       <c r="F2">
-        <v>-1.0707256793975799</v>
+        <v>-0.87937128543853804</v>
       </c>
       <c r="G2">
-        <v>-0.22229230403900099</v>
+        <v>-0.48219949007034302</v>
       </c>
       <c r="H2" t="s">
         <v>38</v>
@@ -10197,7 +10466,7 @@
         <v>39</v>
       </c>
       <c r="K2">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -10211,28 +10480,28 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B3">
-        <v>-9.5861684530973402E-4</v>
+        <v>-1.36055797338486E-3</v>
       </c>
       <c r="C3">
-        <v>3.3118188381195103E-2</v>
+        <v>9.0598642826080295E-2</v>
       </c>
       <c r="D3">
-        <v>-0.20282633602619199</v>
+        <v>-0.17294137179851499</v>
       </c>
       <c r="E3">
-        <v>-0.17964211106300401</v>
+        <v>-9.4194762408733396E-2</v>
       </c>
       <c r="F3">
-        <v>-1.11345994472504</v>
+        <v>-0.93448364734649703</v>
       </c>
       <c r="G3">
-        <v>-0.23012918233871499</v>
+        <v>-0.50216889381408703</v>
       </c>
       <c r="H3" t="s">
         <v>38</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -10246,28 +10515,28 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4">
-        <v>-9.5200352370739005E-4</v>
+        <v>-4.4362898916006099E-4</v>
       </c>
       <c r="C4">
-        <v>3.1913917511701598E-2</v>
+        <v>8.7859079241752597E-2</v>
       </c>
       <c r="D4">
-        <v>-0.185341656208038</v>
+        <v>-0.149700507521629</v>
       </c>
       <c r="E4">
-        <v>-0.159615308046341</v>
+        <v>-8.3662196993827806E-2</v>
       </c>
       <c r="F4">
-        <v>-1.02702784538269</v>
+        <v>-0.81903314590454102</v>
       </c>
       <c r="G4">
-        <v>-0.22407838702201799</v>
+        <v>-0.48939895629882801</v>
       </c>
       <c r="H4" t="s">
         <v>38</v>
       </c>
       <c r="K4">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L4">
         <v>0.6</v>
@@ -10281,28 +10550,28 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5">
-        <v>-2.5325799360871302E-3</v>
+        <v>-2.1755299530923401E-3</v>
       </c>
       <c r="C5">
-        <v>2.99476571381092E-2</v>
+        <v>7.9079501330852495E-2</v>
       </c>
       <c r="D5">
-        <v>-0.19052435457706501</v>
+        <v>-0.15534256398677801</v>
       </c>
       <c r="E5">
-        <v>-0.165864318609238</v>
+        <v>-8.4770120680332198E-2</v>
       </c>
       <c r="F5">
-        <v>-1.05037128925323</v>
+        <v>-0.84200012683868397</v>
       </c>
       <c r="G5">
-        <v>-0.208974063396454</v>
+        <v>-0.437740057706833</v>
       </c>
       <c r="H5" t="s">
         <v>40</v>
       </c>
       <c r="K5">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -12915,22 +13184,22 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37"/>
-      <c r="H1" s="38" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
+      <c r="H1" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="38"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -13820,6 +14089,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E12580AD17ADB64691A1BA4C2E042DA4" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6532fc6a52f3455fe895a4f720bca71c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xmlns:ns4="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9a2f75daf18a7097de825f86ff3fec6" ns3:_="" ns4:_="">
     <xsd:import namespace="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
@@ -14072,14 +14349,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -14090,6 +14359,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65923CC5-95C4-4597-AADE-A0DCE38786F0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14108,23 +14394,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D595912-0053-4104-933F-CDA3B3DBC546}">
   <ds:schemaRefs>

</xml_diff>